<commit_message>
fix: purge leftover template image and enforce zero images on generated BOM sheets
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ITEMS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEMPLATE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RATES" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LISTS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LV453-B61" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PART LIST REFERENCE" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ITEMS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="TEMPLATE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="RATES" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="LISTS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="LV453-B61" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="PART LIST REFERENCE" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -486,39 +486,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>10</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1524000" cy="1524000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20557,7 +20524,6 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: migrate rates column D to active column C, delete column D, add dual IDR/USD tables
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -364,7 +364,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -502,6 +502,9 @@
     </xf>
     <xf numFmtId="3" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5536,7 +5539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T102"/>
+  <dimension ref="A1:U102"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="59" min="1" max="1"/>
@@ -6006,6 +6009,12 @@
           <t>COST IDR (system)</t>
         </is>
       </c>
+      <c r="U17" s="90" t="inlineStr">
+        <is>
+          <t>COST USD
+(system)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
@@ -7012,6 +7021,12 @@
           <t>COST IDR (system)</t>
         </is>
       </c>
+      <c r="U45" s="90" t="inlineStr">
+        <is>
+          <t>COST USD
+(system)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="59">
       <c r="A46" s="9" t="n">
@@ -7044,7 +7059,7 @@
         <f>IF(OR(K46&lt;&gt;"",P46=""),"",1-(IF(H46="",1,H46)*E46*F46)/(ROUNDUP(P46,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R46" s="14">
-        <f>IF(AND(E46="",K46=""),"",IF(B46="","panel type?",IF(AND(K46="",O46=0),"panel bigger than sheet",IF(AND(G46&lt;&gt;"",IFERROR(VALUE(MID(B46,5,FIND("-",B46,5)-5)),0)&lt;&gt;G46),"T must match panel type",IF(I46="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E46="",K46=""),"",IF(B46="","panel type?",IF(AND(K46="",O46=0),"panel bigger than sheet",IF(AND(G46&lt;&gt;"",ISERROR(FIND("-"&amp;G46,B46))),"T must match panel type",IF(I46="","exposed faces?","OK")))))</f>
       </c>
       <c r="S46" s="12">
         <f t="array" ref="S46">IF(OR(B46="",P46=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B46,RATES!$A:$A,0)),"rate?"))</f>
@@ -7084,7 +7099,7 @@
         <f>IF(OR(K47&lt;&gt;"",P47=""),"",1-(IF(H47="",1,H47)*E47*F47)/(ROUNDUP(P47,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R47" s="14">
-        <f>IF(AND(E47="",K47=""),"",IF(B47="","panel type?",IF(AND(K47="",O47=0),"panel bigger than sheet",IF(AND(G47&lt;&gt;"",IFERROR(VALUE(MID(B47,5,FIND("-",B47,5)-5)),0)&lt;&gt;G47),"T must match panel type",IF(I47="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E47="",K47=""),"",IF(B47="","panel type?",IF(AND(K47="",O47=0),"panel bigger than sheet",IF(AND(G47&lt;&gt;"",ISERROR(FIND("-"&amp;G47,B47))),"T must match panel type",IF(I47="","exposed faces?","OK")))))</f>
       </c>
       <c r="S47" s="12">
         <f t="array" ref="S47">IF(OR(B47="",P47=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B47,RATES!$A:$A,0)),"rate?"))</f>
@@ -7124,7 +7139,7 @@
         <f>IF(OR(K48&lt;&gt;"",P48=""),"",1-(IF(H48="",1,H48)*E48*F48)/(ROUNDUP(P48,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R48" s="14">
-        <f>IF(AND(E48="",K48=""),"",IF(B48="","panel type?",IF(AND(K48="",O48=0),"panel bigger than sheet",IF(AND(G48&lt;&gt;"",IFERROR(VALUE(MID(B48,5,FIND("-",B48,5)-5)),0)&lt;&gt;G48),"T must match panel type",IF(I48="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E48="",K48=""),"",IF(B48="","panel type?",IF(AND(K48="",O48=0),"panel bigger than sheet",IF(AND(G48&lt;&gt;"",ISERROR(FIND("-"&amp;G48,B48))),"T must match panel type",IF(I48="","exposed faces?","OK")))))</f>
       </c>
       <c r="S48" s="12">
         <f t="array" ref="S48">IF(OR(B48="",P48=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B48,RATES!$A:$A,0)),"rate?"))</f>
@@ -7164,7 +7179,7 @@
         <f>IF(OR(K49&lt;&gt;"",P49=""),"",1-(IF(H49="",1,H49)*E49*F49)/(ROUNDUP(P49,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R49" s="14">
-        <f>IF(AND(E49="",K49=""),"",IF(B49="","panel type?",IF(AND(K49="",O49=0),"panel bigger than sheet",IF(AND(G49&lt;&gt;"",IFERROR(VALUE(MID(B49,5,FIND("-",B49,5)-5)),0)&lt;&gt;G49),"T must match panel type",IF(I49="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E49="",K49=""),"",IF(B49="","panel type?",IF(AND(K49="",O49=0),"panel bigger than sheet",IF(AND(G49&lt;&gt;"",ISERROR(FIND("-"&amp;G49,B49))),"T must match panel type",IF(I49="","exposed faces?","OK")))))</f>
       </c>
       <c r="S49" s="12">
         <f t="array" ref="S49">IF(OR(B49="",P49=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B49,RATES!$A:$A,0)),"rate?"))</f>
@@ -7204,7 +7219,7 @@
         <f>IF(OR(K50&lt;&gt;"",P50=""),"",1-(IF(H50="",1,H50)*E50*F50)/(ROUNDUP(P50,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R50" s="14">
-        <f>IF(AND(E50="",K50=""),"",IF(B50="","panel type?",IF(AND(K50="",O50=0),"panel bigger than sheet",IF(AND(G50&lt;&gt;"",IFERROR(VALUE(MID(B50,5,FIND("-",B50,5)-5)),0)&lt;&gt;G50),"T must match panel type",IF(I50="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E50="",K50=""),"",IF(B50="","panel type?",IF(AND(K50="",O50=0),"panel bigger than sheet",IF(AND(G50&lt;&gt;"",ISERROR(FIND("-"&amp;G50,B50))),"T must match panel type",IF(I50="","exposed faces?","OK")))))</f>
       </c>
       <c r="S50" s="12">
         <f t="array" ref="S50">IF(OR(B50="",P50=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B50,RATES!$A:$A,0)),"rate?"))</f>
@@ -7244,7 +7259,7 @@
         <f>IF(OR(K51&lt;&gt;"",P51=""),"",1-(IF(H51="",1,H51)*E51*F51)/(ROUNDUP(P51,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R51" s="14">
-        <f>IF(AND(E51="",K51=""),"",IF(B51="","panel type?",IF(AND(K51="",O51=0),"panel bigger than sheet",IF(AND(G51&lt;&gt;"",IFERROR(VALUE(MID(B51,5,FIND("-",B51,5)-5)),0)&lt;&gt;G51),"T must match panel type",IF(I51="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E51="",K51=""),"",IF(B51="","panel type?",IF(AND(K51="",O51=0),"panel bigger than sheet",IF(AND(G51&lt;&gt;"",ISERROR(FIND("-"&amp;G51,B51))),"T must match panel type",IF(I51="","exposed faces?","OK")))))</f>
       </c>
       <c r="S51" s="12">
         <f t="array" ref="S51">IF(OR(B51="",P51=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B51,RATES!$A:$A,0)),"rate?"))</f>
@@ -7284,7 +7299,7 @@
         <f>IF(OR(K52&lt;&gt;"",P52=""),"",1-(IF(H52="",1,H52)*E52*F52)/(ROUNDUP(P52,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R52" s="14">
-        <f>IF(AND(E52="",K52=""),"",IF(B52="","panel type?",IF(AND(K52="",O52=0),"panel bigger than sheet",IF(AND(G52&lt;&gt;"",IFERROR(VALUE(MID(B52,5,FIND("-",B52,5)-5)),0)&lt;&gt;G52),"T must match panel type",IF(I52="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E52="",K52=""),"",IF(B52="","panel type?",IF(AND(K52="",O52=0),"panel bigger than sheet",IF(AND(G52&lt;&gt;"",ISERROR(FIND("-"&amp;G52,B52))),"T must match panel type",IF(I52="","exposed faces?","OK")))))</f>
       </c>
       <c r="S52" s="12">
         <f t="array" ref="S52">IF(OR(B52="",P52=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B52,RATES!$A:$A,0)),"rate?"))</f>
@@ -7324,7 +7339,7 @@
         <f>IF(OR(K53&lt;&gt;"",P53=""),"",1-(IF(H53="",1,H53)*E53*F53)/(ROUNDUP(P53,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R53" s="14">
-        <f>IF(AND(E53="",K53=""),"",IF(B53="","panel type?",IF(AND(K53="",O53=0),"panel bigger than sheet",IF(AND(G53&lt;&gt;"",IFERROR(VALUE(MID(B53,5,FIND("-",B53,5)-5)),0)&lt;&gt;G53),"T must match panel type",IF(I53="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E53="",K53=""),"",IF(B53="","panel type?",IF(AND(K53="",O53=0),"panel bigger than sheet",IF(AND(G53&lt;&gt;"",ISERROR(FIND("-"&amp;G53,B53))),"T must match panel type",IF(I53="","exposed faces?","OK")))))</f>
       </c>
       <c r="S53" s="12">
         <f t="array" ref="S53">IF(OR(B53="",P53=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B53,RATES!$A:$A,0)),"rate?"))</f>
@@ -7364,7 +7379,7 @@
         <f>IF(OR(K54&lt;&gt;"",P54=""),"",1-(IF(H54="",1,H54)*E54*F54)/(ROUNDUP(P54,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R54" s="14">
-        <f>IF(AND(E54="",K54=""),"",IF(B54="","panel type?",IF(AND(K54="",O54=0),"panel bigger than sheet",IF(AND(G54&lt;&gt;"",IFERROR(VALUE(MID(B54,5,FIND("-",B54,5)-5)),0)&lt;&gt;G54),"T must match panel type",IF(I54="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E54="",K54=""),"",IF(B54="","panel type?",IF(AND(K54="",O54=0),"panel bigger than sheet",IF(AND(G54&lt;&gt;"",ISERROR(FIND("-"&amp;G54,B54))),"T must match panel type",IF(I54="","exposed faces?","OK")))))</f>
       </c>
       <c r="S54" s="12">
         <f t="array" ref="S54">IF(OR(B54="",P54=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B54,RATES!$A:$A,0)),"rate?"))</f>
@@ -7404,7 +7419,7 @@
         <f>IF(OR(K55&lt;&gt;"",P55=""),"",1-(IF(H55="",1,H55)*E55*F55)/(ROUNDUP(P55,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R55" s="14">
-        <f>IF(AND(E55="",K55=""),"",IF(B55="","panel type?",IF(AND(K55="",O55=0),"panel bigger than sheet",IF(AND(G55&lt;&gt;"",IFERROR(VALUE(MID(B55,5,FIND("-",B55,5)-5)),0)&lt;&gt;G55),"T must match panel type",IF(I55="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E55="",K55=""),"",IF(B55="","panel type?",IF(AND(K55="",O55=0),"panel bigger than sheet",IF(AND(G55&lt;&gt;"",ISERROR(FIND("-"&amp;G55,B55))),"T must match panel type",IF(I55="","exposed faces?","OK")))))</f>
       </c>
       <c r="S55" s="12">
         <f t="array" ref="S55">IF(OR(B55="",P55=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B55,RATES!$A:$A,0)),"rate?"))</f>
@@ -7444,7 +7459,7 @@
         <f>IF(OR(K56&lt;&gt;"",P56=""),"",1-(IF(H56="",1,H56)*E56*F56)/(ROUNDUP(P56,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R56" s="14">
-        <f>IF(AND(E56="",K56=""),"",IF(B56="","panel type?",IF(AND(K56="",O56=0),"panel bigger than sheet",IF(AND(G56&lt;&gt;"",IFERROR(VALUE(MID(B56,5,FIND("-",B56,5)-5)),0)&lt;&gt;G56),"T must match panel type",IF(I56="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E56="",K56=""),"",IF(B56="","panel type?",IF(AND(K56="",O56=0),"panel bigger than sheet",IF(AND(G56&lt;&gt;"",ISERROR(FIND("-"&amp;G56,B56))),"T must match panel type",IF(I56="","exposed faces?","OK")))))</f>
       </c>
       <c r="S56" s="12">
         <f t="array" ref="S56">IF(OR(B56="",P56=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B56,RATES!$A:$A,0)),"rate?"))</f>
@@ -7484,7 +7499,7 @@
         <f>IF(OR(K57&lt;&gt;"",P57=""),"",1-(IF(H57="",1,H57)*E57*F57)/(ROUNDUP(P57,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R57" s="14">
-        <f>IF(AND(E57="",K57=""),"",IF(B57="","panel type?",IF(AND(K57="",O57=0),"panel bigger than sheet",IF(AND(G57&lt;&gt;"",IFERROR(VALUE(MID(B57,5,FIND("-",B57,5)-5)),0)&lt;&gt;G57),"T must match panel type",IF(I57="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E57="",K57=""),"",IF(B57="","panel type?",IF(AND(K57="",O57=0),"panel bigger than sheet",IF(AND(G57&lt;&gt;"",ISERROR(FIND("-"&amp;G57,B57))),"T must match panel type",IF(I57="","exposed faces?","OK")))))</f>
       </c>
       <c r="S57" s="12">
         <f t="array" ref="S57">IF(OR(B57="",P57=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B57,RATES!$A:$A,0)),"rate?"))</f>
@@ -7524,7 +7539,7 @@
         <f>IF(OR(K58&lt;&gt;"",P58=""),"",1-(IF(H58="",1,H58)*E58*F58)/(ROUNDUP(P58,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R58" s="14">
-        <f>IF(AND(E58="",K58=""),"",IF(B58="","panel type?",IF(AND(K58="",O58=0),"panel bigger than sheet",IF(AND(G58&lt;&gt;"",IFERROR(VALUE(MID(B58,5,FIND("-",B58,5)-5)),0)&lt;&gt;G58),"T must match panel type",IF(I58="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E58="",K58=""),"",IF(B58="","panel type?",IF(AND(K58="",O58=0),"panel bigger than sheet",IF(AND(G58&lt;&gt;"",ISERROR(FIND("-"&amp;G58,B58))),"T must match panel type",IF(I58="","exposed faces?","OK")))))</f>
       </c>
       <c r="S58" s="12">
         <f t="array" ref="S58">IF(OR(B58="",P58=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B58,RATES!$A:$A,0)),"rate?"))</f>
@@ -7564,7 +7579,7 @@
         <f>IF(OR(K59&lt;&gt;"",P59=""),"",1-(IF(H59="",1,H59)*E59*F59)/(ROUNDUP(P59,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R59" s="14">
-        <f>IF(AND(E59="",K59=""),"",IF(B59="","panel type?",IF(AND(K59="",O59=0),"panel bigger than sheet",IF(AND(G59&lt;&gt;"",IFERROR(VALUE(MID(B59,5,FIND("-",B59,5)-5)),0)&lt;&gt;G59),"T must match panel type",IF(I59="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E59="",K59=""),"",IF(B59="","panel type?",IF(AND(K59="",O59=0),"panel bigger than sheet",IF(AND(G59&lt;&gt;"",ISERROR(FIND("-"&amp;G59,B59))),"T must match panel type",IF(I59="","exposed faces?","OK")))))</f>
       </c>
       <c r="S59" s="12">
         <f t="array" ref="S59">IF(OR(B59="",P59=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B59,RATES!$A:$A,0)),"rate?"))</f>
@@ -7604,7 +7619,7 @@
         <f>IF(OR(K60&lt;&gt;"",P60=""),"",1-(IF(H60="",1,H60)*E60*F60)/(ROUNDUP(P60,0)*LISTS!$F$6*LISTS!$F$7))</f>
       </c>
       <c r="R60" s="14">
-        <f>IF(AND(E60="",K60=""),"",IF(B60="","panel type?",IF(AND(K60="",O60=0),"panel bigger than sheet",IF(AND(G60&lt;&gt;"",IFERROR(VALUE(MID(B60,5,FIND("-",B60,5)-5)),0)&lt;&gt;G60),"T must match panel type",IF(I60="","exposed faces?","OK")))))</f>
+        <f>IF(AND(E60="",K60=""),"",IF(B60="","panel type?",IF(AND(K60="",O60=0),"panel bigger than sheet",IF(AND(G60&lt;&gt;"",ISERROR(FIND("-"&amp;G60,B60))),"T must match panel type",IF(I60="","exposed faces?","OK")))))</f>
       </c>
       <c r="S60" s="12">
         <f t="array" ref="S60">IF(OR(B60="",P60=""),"",IFERROR(INDEX(RATES!$C:$C,MATCH(B60,RATES!$A:$A,0)),"rate?"))</f>
@@ -7680,6 +7695,11 @@
       <c r="T63" s="8" t="inlineStr">
         <is>
           <t>LINE TOTAL (calc)</t>
+        </is>
+      </c>
+      <c r="U63" s="90" t="inlineStr">
+        <is>
+          <t>LINE TOTAL USD</t>
         </is>
       </c>
     </row>
@@ -8079,6 +8099,11 @@
       <c r="A81" s="5" t="inlineStr">
         <is>
           <t>SUMMARY (system): cost per ONE item, from the RATES tab. Do not type here.</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>COST USD (system)</t>
         </is>
       </c>
     </row>
@@ -9340,7 +9365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J229"/>
+  <dimension ref="A1:J249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10101,12 +10126,10 @@
           <t>Carpentry labour per m³ of component (inside every tier rate)</t>
         </is>
       </c>
-      <c r="C34" s="81">
-        <f>$C$10*(1-$C$11)/$C$12</f>
-      </c>
-      <c r="D34" s="81" t="n">
+      <c r="C34" s="81" t="n">
         <v>4000000</v>
       </c>
+      <c r="D34" s="81" t="n"/>
       <c r="E34" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10129,12 +10152,10 @@
           <t>Teak tier A</t>
         </is>
       </c>
-      <c r="C35" s="81">
-        <f>($C$6+$C$9)*$C$13+$C$34</f>
-      </c>
-      <c r="D35" s="81">
-        <f>C35*0.9</f>
-      </c>
+      <c r="C35" s="81" t="n">
+        <v>27507965.09</v>
+      </c>
+      <c r="D35" s="81" t="n"/>
       <c r="E35" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10157,12 +10178,10 @@
           <t>Teak tier A-CURVED</t>
         </is>
       </c>
-      <c r="C36" s="81">
-        <f>($C$6+$C$9)*$C$14+$C$34</f>
-      </c>
-      <c r="D36" s="81">
-        <f>C36*0.9</f>
-      </c>
+      <c r="C36" s="81" t="n">
+        <v>34040953.31</v>
+      </c>
+      <c r="D36" s="81" t="n"/>
       <c r="E36" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10180,12 +10199,10 @@
           <t>Teak tier B</t>
         </is>
       </c>
-      <c r="C37" s="81">
-        <f>($C$6+$C$9)*$C$15+$C$34</f>
-      </c>
-      <c r="D37" s="81">
-        <f>C37*0.9</f>
-      </c>
+      <c r="C37" s="81" t="n">
+        <v>21568884.89</v>
+      </c>
+      <c r="D37" s="81" t="n"/>
       <c r="E37" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10203,12 +10220,10 @@
           <t>Teak tier C</t>
         </is>
       </c>
-      <c r="C38" s="81">
-        <f>($C$6+$C$9)*$C$16+$C$34</f>
-      </c>
-      <c r="D38" s="81">
-        <f>C38*0.9</f>
-      </c>
+      <c r="C38" s="81" t="n">
+        <v>18599344.79</v>
+      </c>
+      <c r="D38" s="81" t="n"/>
       <c r="E38" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10226,12 +10241,10 @@
           <t>Teak tier D</t>
         </is>
       </c>
-      <c r="C39" s="81">
-        <f>($C$6+$C$9)*$C$17+$C$34</f>
-      </c>
-      <c r="D39" s="81">
-        <f>C39*0.9</f>
-      </c>
+      <c r="C39" s="81" t="n">
+        <v>15629804.69</v>
+      </c>
+      <c r="D39" s="81" t="n"/>
       <c r="E39" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10249,12 +10262,10 @@
           <t>Mindi tier A</t>
         </is>
       </c>
-      <c r="C40" s="81">
-        <f>($C$7+$C$9)*$C$13+$C$34</f>
-      </c>
-      <c r="D40" s="81">
-        <f>C40*0.9</f>
-      </c>
+      <c r="C40" s="81" t="n">
+        <v>18057965.09</v>
+      </c>
+      <c r="D40" s="81" t="n"/>
       <c r="E40" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10272,12 +10283,10 @@
           <t>Mindi tier A-CURVED</t>
         </is>
       </c>
-      <c r="C41" s="81">
-        <f>($C$7+$C$9)*$C$14+$C$34</f>
-      </c>
-      <c r="D41" s="81">
-        <f>C41*0.9</f>
-      </c>
+      <c r="C41" s="81" t="n">
+        <v>21620953.31</v>
+      </c>
+      <c r="D41" s="81" t="n"/>
       <c r="E41" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10295,12 +10304,10 @@
           <t>Mindi tier B</t>
         </is>
       </c>
-      <c r="C42" s="81">
-        <f>($C$7+$C$9)*$C$15+$C$34</f>
-      </c>
-      <c r="D42" s="81">
-        <f>C42*0.9</f>
-      </c>
+      <c r="C42" s="81" t="n">
+        <v>14818884.89</v>
+      </c>
+      <c r="D42" s="81" t="n"/>
       <c r="E42" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10318,12 +10325,10 @@
           <t>Mindi tier C</t>
         </is>
       </c>
-      <c r="C43" s="81">
-        <f>($C$7+$C$9)*$C$16+$C$34</f>
-      </c>
-      <c r="D43" s="81">
-        <f>C43*0.9</f>
-      </c>
+      <c r="C43" s="81" t="n">
+        <v>13199344.79</v>
+      </c>
+      <c r="D43" s="81" t="n"/>
       <c r="E43" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10341,12 +10346,10 @@
           <t>Mindi tier D</t>
         </is>
       </c>
-      <c r="C44" s="81">
-        <f>($C$7+$C$9)*$C$17+$C$34</f>
-      </c>
-      <c r="D44" s="81">
-        <f>C44*0.9</f>
-      </c>
+      <c r="C44" s="81" t="n">
+        <v>11579804.69</v>
+      </c>
+      <c r="D44" s="81" t="n"/>
       <c r="E44" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10364,12 +10367,10 @@
           <t>Meranti, any tier</t>
         </is>
       </c>
-      <c r="C45" s="81">
-        <f>$C$8*$C$18+$C$34</f>
-      </c>
-      <c r="D45" s="81">
-        <f>C45*0.9</f>
-      </c>
+      <c r="C45" s="81" t="n">
+        <v>18196184.39</v>
+      </c>
+      <c r="D45" s="81" t="n"/>
       <c r="E45" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10392,12 +10393,10 @@
           <t>Screws, nails, dowels, glue per m³ of component</t>
         </is>
       </c>
-      <c r="C46" s="81">
-        <f>$C$19/$C$12</f>
-      </c>
-      <c r="D46" s="81" t="n">
+      <c r="C46" s="81" t="n">
         <v>1000000</v>
       </c>
+      <c r="D46" s="81" t="n"/>
       <c r="E46" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10415,12 +10414,10 @@
           <t>Finishing materials (Zhanchen + thinner) per m² exposed</t>
         </is>
       </c>
-      <c r="C47" s="81">
-        <f>$C$20/$C$25</f>
-      </c>
-      <c r="D47" s="81" t="n">
+      <c r="C47" s="81" t="n">
         <v>37000</v>
       </c>
+      <c r="D47" s="81" t="n"/>
       <c r="E47" s="74" t="inlineStr">
         <is>
           <t>IDR/m²</t>
@@ -10438,12 +10435,10 @@
           <t>Sanding materials (abrasives) per m² exposed</t>
         </is>
       </c>
-      <c r="C48" s="81">
-        <f>$C$21/$C$25</f>
-      </c>
-      <c r="D48" s="81">
-        <f>C48*0.8</f>
-      </c>
+      <c r="C48" s="81" t="n">
+        <v>10235.64174</v>
+      </c>
+      <c r="D48" s="81" t="n"/>
       <c r="E48" s="74" t="inlineStr">
         <is>
           <t>IDR/m²</t>
@@ -10461,12 +10456,10 @@
           <t>Sanding labour (65% of sanding pool) per m² exposed</t>
         </is>
       </c>
-      <c r="C49" s="81">
-        <f>$C$23*$C$24/$C$25</f>
-      </c>
-      <c r="D49" s="81" t="n">
+      <c r="C49" s="81" t="n">
         <v>20000</v>
       </c>
+      <c r="D49" s="81" t="n"/>
       <c r="E49" s="74" t="inlineStr">
         <is>
           <t>IDR/m²</t>
@@ -10484,12 +10477,10 @@
           <t>Finishing labour (finishing pool) per m² exposed</t>
         </is>
       </c>
-      <c r="C50" s="81">
-        <f>$C$22/$C$25</f>
-      </c>
-      <c r="D50" s="81" t="n">
+      <c r="C50" s="81" t="n">
         <v>45000</v>
       </c>
+      <c r="D50" s="81" t="n"/>
       <c r="E50" s="74" t="inlineStr">
         <is>
           <t>IDR/m²</t>
@@ -10508,11 +10499,9 @@
         </is>
       </c>
       <c r="C51" s="80" t="n">
-        <v>42000</v>
-      </c>
-      <c r="D51" s="80" t="n">
         <v>40000</v>
       </c>
+      <c r="D51" s="80" t="n"/>
       <c r="E51" s="74" t="inlineStr">
         <is>
           <t>IDR/m²</t>
@@ -10536,11 +10525,9 @@
         </is>
       </c>
       <c r="C52" s="80" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D52" s="80" t="n">
         <v>50000</v>
       </c>
+      <c r="D52" s="80" t="n"/>
       <c r="E52" s="74" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -10665,12 +10652,10 @@
           <t>Mindi veneer added cost per face</t>
         </is>
       </c>
-      <c r="C58" s="81">
-        <f>$C$30*$C$31+$C$28*(LISTS!$F$6*LISTS!$F$7/1000000)+$C$32</f>
-      </c>
-      <c r="D58" s="81" t="n">
+      <c r="C58" s="81" t="n">
         <v>18000</v>
       </c>
+      <c r="D58" s="81" t="n"/>
       <c r="E58" s="74" t="inlineStr">
         <is>
           <t>m2</t>
@@ -12945,6 +12930,7 @@
         </is>
       </c>
     </row>
+    <row r="169"/>
     <row r="170">
       <c r="A170" s="84" t="inlineStr">
         <is>
@@ -13126,6 +13112,7 @@
         </is>
       </c>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="79" t="inlineStr">
         <is>
@@ -14532,6 +14519,7 @@
         <v>933</v>
       </c>
     </row>
+    <row r="216"/>
     <row r="217">
       <c r="A217" s="84" t="inlineStr">
         <is>
@@ -14787,6 +14775,7 @@
         <f>G225*$C$172</f>
       </c>
     </row>
+    <row r="226"/>
     <row r="227">
       <c r="A227" s="84" t="inlineStr">
         <is>
@@ -14864,6 +14853,374 @@
       </c>
       <c r="H229" s="83">
         <f>G229*$C$172</f>
+      </c>
+    </row>
+    <row r="230"/>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>VENEERED LANDED BOARDS (E2 + Mindi Veneer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MSF</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Plywood E2 18 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C232">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-18",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MDF</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Plywood E2 18 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C233">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-18",$A$178:$A$215,0))+2*$C$175</f>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MSF</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Plywood E2 15 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C234">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-15",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MDF</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Plywood E2 15 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C235">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-15",$A$178:$A$215,0))+2*$C$175</f>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MSF</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Plywood E2 12 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C236">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-12",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MDF</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Plywood E2 12 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C237">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-12",$A$178:$A$215,0))+2*$C$175</f>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MSF</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Plywood E2 9 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C238">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-9",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MDF</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Plywood E2 9 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C239">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-9",$A$178:$A$215,0))+2*$C$175</f>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MSF</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Plywood E2 6 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C240">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-6",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MDF</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Plywood E2 6 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C241">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-6",$A$178:$A$215,0))+2*$C$175</f>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MSF</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Plywood E2 3 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C242">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-3",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MDF</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Plywood E2 3 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C243">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E2-3",$A$178:$A$215,0))+2*$C$175</f>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MSF</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>MDF E2 18 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C244">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E2-18",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MDF</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>MDF E2 18 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C245">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E2-18",$A$178:$A$215,0))+2*$C$175</f>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-15-MSF</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>MDF E2 15 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C246">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E2-15",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-12-MSF</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>MDF E2 12 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C247">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E2-12",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-9-MSF</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>MDF E2 9 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C248">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E2-9",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-6-MSF</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>MDF E2 6 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C249">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E2-6",$A$178:$A$215,0))+$C$175</f>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(rules): lock ALL plywood and MDF to grade E2 (config, rate card, checker rejects E0/CARB, tests)
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -11790,7 +11790,7 @@
       </c>
       <c r="E59" s="96" t="inlineStr">
         <is>
-          <t>Mojo Indah list, Sep 2026</t>
+          <t>E2 landed Kudus (Linyi quote 16 Oct 2026). Grade LOCKED E2</t>
         </is>
       </c>
       <c r="F59" s="112">
@@ -11930,7 +11930,7 @@
       </c>
       <c r="E64" s="96" t="inlineStr">
         <is>
-          <t>Mojo Indah list, Sep 2026</t>
+          <t>E2 landed Kudus (Linyi quote 16 Oct 2026). Grade LOCKED E2</t>
         </is>
       </c>
       <c r="F64" s="112">
@@ -12070,7 +12070,7 @@
       </c>
       <c r="E69" s="96" t="inlineStr">
         <is>
-          <t>Mojo Indah list, Sep 2026</t>
+          <t>E2 landed Kudus (Linyi quote 16 Oct 2026). Grade LOCKED E2</t>
         </is>
       </c>
       <c r="F69" s="112">
@@ -12210,7 +12210,7 @@
       </c>
       <c r="E74" s="96" t="inlineStr">
         <is>
-          <t>Mojo Indah list, Sep 2026</t>
+          <t>E2 landed Kudus (Linyi quote 16 Oct 2026). Grade LOCKED E2</t>
         </is>
       </c>
       <c r="F74" s="112">
@@ -12349,7 +12349,7 @@
       </c>
       <c r="E79" s="96" t="inlineStr">
         <is>
-          <t>Mojo Indah list, Sep 2026</t>
+          <t>E2 landed Kudus (Linyi quote 16 Oct 2026). Grade LOCKED E2</t>
         </is>
       </c>
       <c r="F79" s="112">
@@ -12485,7 +12485,7 @@
       </c>
       <c r="E84" s="96" t="inlineStr">
         <is>
-          <t>Mojo Indah list, Sep 2026</t>
+          <t>E2 landed Kudus (Linyi quote 16 Oct 2026). Grade LOCKED E2</t>
         </is>
       </c>
       <c r="F84" s="112">
@@ -14734,7 +14734,7 @@
       </c>
       <c r="B174" s="117" t="inlineStr">
         <is>
-          <t>Board grade feeding the PLY-x and MDF-x rates (type E2, E0 or CARB)</t>
+          <t>Board grade for ALL plywood and MDF (LOCKED E2, rule 19 Oct 2026). Do not change.</t>
         </is>
       </c>
       <c r="C174" s="118" t="inlineStr">
@@ -14749,7 +14749,7 @@
       </c>
       <c r="E174" s="113" t="inlineStr">
         <is>
-          <t>CARB Phase 2 / TSCA Title VI: required for US hotel projects, accepted for EU</t>
+          <t>Rule: plywood (B group) and MDF (C group) always E2, landed Kudus. E0 / CARB rows are reference only.</t>
         </is>
       </c>
       <c r="F174" s="95" t="n"/>

</xml_diff>

<commit_message>
feat(rules): all panels use explicit E2 codes (LND-PLY-E2-*, LND-MDF-E2-*); auto-normalise legacy codes; specs, LISTS dropdown, tests updated
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -17407,7 +17407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="16" customWidth="1" style="59" min="1" max="2"/>
@@ -17465,7 +17465,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>PLY-3-RAW</t>
+          <t>LND-PLY-E2-3</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -17495,7 +17495,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>PLY-3-MSF</t>
+          <t>LND-PLY-E2-6</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -17525,7 +17525,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>PLY-3-MDF</t>
+          <t>LND-PLY-E2-9</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -17550,7 +17550,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>PLY-3-TSF</t>
+          <t>LND-PLY-E2-12</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -17570,7 +17570,7 @@
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PLY-3-TDF</t>
+          <t>LND-PLY-E2-15</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -17590,7 +17590,7 @@
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PLY-6-RAW</t>
+          <t>LND-PLY-E2-18</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -17605,7 +17605,7 @@
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>PLY-6-MSF</t>
+          <t>LND-MDF-E2-3</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -17620,7 +17620,7 @@
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PLY-6-MDF</t>
+          <t>LND-MDF-E2-6</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -17635,7 +17635,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PLY-6-TSF</t>
+          <t>LND-MDF-E2-9</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -17650,184 +17650,164 @@
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PLY-6-TDF</t>
+          <t>LND-MDF-E2-12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PLY-9-RAW</t>
+          <t>LND-MDF-E2-15</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PLY-9-MSF</t>
+          <t>LND-MDF-E2-18</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PLY-9-MDF</t>
+          <t>LND-PLY-E2-18-MSF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>PLY-9-TSF</t>
+          <t>LND-PLY-E2-18-MDF</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PLY-9-TDF</t>
+          <t>LND-PLY-E2-15-MSF</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>PLY-12-RAW</t>
+          <t>LND-PLY-E2-15-MDF</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>PLY-12-MSF</t>
+          <t>LND-PLY-E2-12-MSF</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PLY-12-MDF</t>
+          <t>LND-PLY-E2-12-MDF</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="59">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>PLY-12-TSF</t>
+          <t>LND-PLY-E2-9-MSF</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="59">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>PLY-12-TDF</t>
+          <t>LND-PLY-E2-9-MDF</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="59">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>PLY-15-RAW</t>
+          <t>LND-PLY-E2-6-MSF</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="59">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>PLY-15-MSF</t>
+          <t>LND-PLY-E2-6-MDF</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="59">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>PLY-15-MDF</t>
+          <t>LND-PLY-E2-3-MSF</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="59">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>PLY-15-TSF</t>
+          <t>LND-PLY-E2-3-MDF</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="59">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>PLY-15-TDF</t>
+          <t>LND-MDF-E2-18-MSF</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="59">
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>PLY-18-RAW</t>
+          <t>LND-MDF-E2-18-MDF</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="59">
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PLY-18-MSF</t>
+          <t>LND-MDF-E2-15-MSF</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="59">
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>PLY-18-MDF</t>
+          <t>LND-MDF-E2-12-MSF</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="59">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>PLY-18-TSF</t>
+          <t>LND-MDF-E2-9-MSF</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="59">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>PLY-18-TDF</t>
+          <t>LND-MDF-E2-6-MSF</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="59">
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>PLY-24-RAW</t>
-        </is>
-      </c>
+      <c r="B33" s="2" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="59">
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>PLY-24-MSF</t>
-        </is>
-      </c>
+      <c r="B34" s="2" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="59">
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>PLY-24-MDF</t>
-        </is>
-      </c>
+      <c r="B35" s="2" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="59">
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>PLY-24-TSF</t>
-        </is>
-      </c>
+      <c r="B36" s="2" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="59">
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>PLY-24-TDF</t>
-        </is>
-      </c>
+      <c r="B37" s="2" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="59"/>
     <row r="39" ht="15.75" customHeight="1" s="59"/>

</xml_diff>

<commit_message>
feat(layout): auto-highlight missing prices (conditional formatting) on item sheets and RATES
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -642,6 +642,20 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C2B00"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7A0"/>
+          <bgColor rgb="00FFC7A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -10185,6 +10199,21 @@
     <mergeCell ref="L76:R76"/>
     <mergeCell ref="D6:F6"/>
   </mergeCells>
+  <conditionalFormatting sqref="S18:T42">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND($E18&lt;&gt;"",OR(S18="",S18=0,S18="rate?"))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S46:T60">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
+      <formula>AND($E46&lt;&gt;"",OR(S46="",S46=0,S46="rate?"))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S64:T78">
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="0">
+      <formula>AND($D64&lt;&gt;"",OR(S64="",S64=0))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation sqref="K18:K42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A,A-CURVED,B,C,D"</formula1>
@@ -14605,7 +14634,6 @@
       <c r="H168" s="95" t="n"/>
       <c r="I168" s="95" t="n"/>
     </row>
-    <row r="169"/>
     <row r="170">
       <c r="A170" s="97" t="inlineStr">
         <is>
@@ -14815,7 +14843,6 @@
       <c r="H176" s="95" t="n"/>
       <c r="I176" s="95" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="119" t="inlineStr">
         <is>
@@ -16336,7 +16363,6 @@
         <v>933</v>
       </c>
     </row>
-    <row r="216"/>
     <row r="217">
       <c r="A217" s="97" t="inlineStr">
         <is>
@@ -16640,7 +16666,6 @@
       <c r="H225" s="95" t="n"/>
       <c r="I225" s="95" t="n"/>
     </row>
-    <row r="226"/>
     <row r="227">
       <c r="A227" s="97" t="inlineStr">
         <is>
@@ -16734,7 +16759,6 @@
       <c r="H229" s="95" t="n"/>
       <c r="I229" s="95" t="n"/>
     </row>
-    <row r="230"/>
     <row r="231">
       <c r="A231" s="127" t="inlineStr">
         <is>
@@ -17218,7 +17242,6 @@
       <c r="H249" s="95" t="n"/>
       <c r="I249" s="95" t="n"/>
     </row>
-    <row r="250"/>
     <row r="251">
       <c r="A251" s="127" t="inlineStr">
         <is>
@@ -17397,6 +17420,11 @@
       <c r="I257" s="95" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C5:C400">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>AND($A5&lt;&gt;"",$A5&lt;&gt;"code",$B5&lt;&gt;"",$C5="")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17407,7 +17435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="16" customWidth="1" style="59" min="1" max="2"/>

</xml_diff>

<commit_message>
feat(rules): curve rule (R30/R40 rounded corners): A-CURVED tier, blank = finished + arc + CURVE_ALLOW; model radius/corners; RATES CURVE_ALLOW (empty); B41 tagged; tests
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -10239,7 +10239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I257"/>
+  <dimension ref="A1:I260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="59" min="1" max="1"/>
@@ -14634,6 +14634,7 @@
       <c r="H168" s="95" t="n"/>
       <c r="I168" s="95" t="n"/>
     </row>
+    <row r="169"/>
     <row r="170">
       <c r="A170" s="97" t="inlineStr">
         <is>
@@ -14843,6 +14844,7 @@
       <c r="H176" s="95" t="n"/>
       <c r="I176" s="95" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="119" t="inlineStr">
         <is>
@@ -16363,6 +16365,7 @@
         <v>933</v>
       </c>
     </row>
+    <row r="216"/>
     <row r="217">
       <c r="A217" s="97" t="inlineStr">
         <is>
@@ -16666,6 +16669,7 @@
       <c r="H225" s="95" t="n"/>
       <c r="I225" s="95" t="n"/>
     </row>
+    <row r="226"/>
     <row r="227">
       <c r="A227" s="97" t="inlineStr">
         <is>
@@ -16759,6 +16763,7 @@
       <c r="H229" s="95" t="n"/>
       <c r="I229" s="95" t="n"/>
     </row>
+    <row r="230"/>
     <row r="231">
       <c r="A231" s="127" t="inlineStr">
         <is>
@@ -17242,6 +17247,7 @@
       <c r="H249" s="95" t="n"/>
       <c r="I249" s="95" t="n"/>
     </row>
+    <row r="250"/>
     <row r="251">
       <c r="A251" s="127" t="inlineStr">
         <is>
@@ -17418,6 +17424,41 @@
       <c r="G257" s="95" t="n"/>
       <c r="H257" s="95" t="n"/>
       <c r="I257" s="95" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="127" t="inlineStr">
+        <is>
+          <t>CURVES (added 19 Oct 2026). Rounded corners R30/R40: tier A-CURVED, blank = finished + arc + tolerance. Value EMPTY until factory gives the tolerance.</t>
+        </is>
+      </c>
+      <c r="B259" s="98" t="n"/>
+      <c r="C259" s="98" t="n"/>
+      <c r="D259" s="98" t="n"/>
+      <c r="E259" s="98" t="n"/>
+      <c r="F259" s="98" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="113" t="inlineStr">
+        <is>
+          <t>CURVE_ALLOW</t>
+        </is>
+      </c>
+      <c r="B260" s="117" t="inlineStr">
+        <is>
+          <t>Tolerance added to length and width of a curved part (arc is computed from the radius)</t>
+        </is>
+      </c>
+      <c r="C260" s="129" t="n"/>
+      <c r="D260" s="113" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E260" s="113" t="inlineStr">
+        <is>
+          <t>EMPTY: waiting for factory figure</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5:C400">

</xml_diff>

<commit_message>
feat(veneer): veneer cost from log price, yield and slicing fee for 0.6/1.0/1.2 mm (default 0.6; -V10/-V12 codes); RATES block + config; missing panel code now errors; tests
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -10239,7 +10239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I260"/>
+  <dimension ref="A1:I315"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="59" min="1" max="1"/>
@@ -14797,8 +14797,9 @@
           <t>Mindi veneer added per face inside the PLY-x-MSF / MDF rates</t>
         </is>
       </c>
-      <c r="C175" s="114" t="n">
-        <v>147709.02</v>
+      <c r="C175" s="114">
+        <f>C275</f>
+        <v/>
       </c>
       <c r="D175" s="113" t="inlineStr">
         <is>
@@ -14807,7 +14808,7 @@
       </c>
       <c r="E175" s="113" t="inlineStr">
         <is>
-          <t>Back-calculated from the 29 Sep rate card (PLY-x-MSF minus PLY-x-RAW). Not the same as VEN_MINDI_FACE.</t>
+          <t>Now a formula: 0.6 mm face from the VENEER block below (was fixed 147,709).</t>
         </is>
       </c>
       <c r="F175" s="95" t="n"/>
@@ -17425,6 +17426,7 @@
       <c r="H257" s="95" t="n"/>
       <c r="I257" s="95" t="n"/>
     </row>
+    <row r="258"/>
     <row r="259">
       <c r="A259" s="127" t="inlineStr">
         <is>
@@ -17459,6 +17461,1386 @@
           <t>EMPTY: waiting for factory figure</t>
         </is>
       </c>
+    </row>
+    <row r="261"/>
+    <row r="262">
+      <c r="A262" s="127" t="inlineStr">
+        <is>
+          <t>VENEER (added 19 Oct 2026). Face veneer cost is built from log price, slicing yield and vendor fee, for 0.6 / 1.0 / 1.2 mm. Default board codes (-MSF, -MDF) use 0.6 mm. Add -V10 or -V12 to the code for 1.0 or 1.2 mm.</t>
+        </is>
+      </c>
+      <c r="B262" s="98" t="n"/>
+      <c r="C262" s="98" t="n"/>
+      <c r="D262" s="98" t="n"/>
+      <c r="E262" s="98" t="n"/>
+      <c r="F262" s="98" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="113" t="inlineStr">
+        <is>
+          <t>VEN_LOG_PRICE</t>
+        </is>
+      </c>
+      <c r="B263" s="117" t="inlineStr">
+        <is>
+          <t>Mindi log price for veneer</t>
+        </is>
+      </c>
+      <c r="C263" s="129" t="n">
+        <v>3200000</v>
+      </c>
+      <c r="D263" s="113" t="inlineStr">
+        <is>
+          <t>IDR/m³</t>
+        </is>
+      </c>
+      <c r="E263" s="113" t="inlineStr">
+        <is>
+          <t>Update 19 Oct 2026. Status CONFIRM (log_mindi in this card is 3,000,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="113" t="inlineStr">
+        <is>
+          <t>VEN_SLICE_YIELD</t>
+        </is>
+      </c>
+      <c r="B264" s="117" t="inlineStr">
+        <is>
+          <t>Slicing yield quoted by the veneer vendor</t>
+        </is>
+      </c>
+      <c r="C264" s="129" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D264" s="113" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E264" s="113" t="inlineStr">
+        <is>
+          <t>Vendor, mindi / mahogany. Status CONFIRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="113" t="inlineStr">
+        <is>
+          <t>VEN_FLITCH_W</t>
+        </is>
+      </c>
+      <c r="B265" s="117" t="inlineStr">
+        <is>
+          <t>Flitch width before trimming</t>
+        </is>
+      </c>
+      <c r="C265" s="129" t="n">
+        <v>160</v>
+      </c>
+      <c r="D265" s="113" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E265" s="113" t="inlineStr">
+        <is>
+          <t>Vendor flitch 2.5 m long</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="113" t="inlineStr">
+        <is>
+          <t>VEN_TRIM_W</t>
+        </is>
+      </c>
+      <c r="B266" s="117" t="inlineStr">
+        <is>
+          <t>Flitch width after trimming</t>
+        </is>
+      </c>
+      <c r="C266" s="129" t="n">
+        <v>150</v>
+      </c>
+      <c r="D266" s="113" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E266" s="113" t="inlineStr">
+        <is>
+          <t>Vendor flitch 2.5 m long</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="113" t="inlineStr">
+        <is>
+          <t>VEN_YIELD_EFF</t>
+        </is>
+      </c>
+      <c r="B267" s="117" t="inlineStr">
+        <is>
+          <t>Effective yield = slicing yield x trim width / flitch width</t>
+        </is>
+      </c>
+      <c r="C267" s="129">
+        <f>C264*C266/C265</f>
+        <v/>
+      </c>
+      <c r="D267" s="113" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E267" s="113" t="inlineStr">
+        <is>
+          <t>Formula (28.125% with the figures above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="113" t="inlineStr">
+        <is>
+          <t>VEN_SLICE_FEE</t>
+        </is>
+      </c>
+      <c r="B268" s="117" t="inlineStr">
+        <is>
+          <t>Slicing fee, per m2 of usable veneer</t>
+        </is>
+      </c>
+      <c r="C268" s="129" t="n">
+        <v>12000</v>
+      </c>
+      <c r="D268" s="113" t="inlineStr">
+        <is>
+          <t>IDR/m²</t>
+        </is>
+      </c>
+      <c r="E268" s="113" t="inlineStr">
+        <is>
+          <t>Vendor. Matches market 0.6 mm at 18-20 ribu. Status CONFIRM (assumed billed on usable m2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="113" t="inlineStr">
+        <is>
+          <t>VEN_T_06</t>
+        </is>
+      </c>
+      <c r="B269" s="117" t="inlineStr">
+        <is>
+          <t>Veneer thickness 0.6 mm</t>
+        </is>
+      </c>
+      <c r="C269" s="129" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D269" s="113" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E269" s="113" t="inlineStr">
+        <is>
+          <t>Industry sliced thickness</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="113" t="inlineStr">
+        <is>
+          <t>VEN_T_10</t>
+        </is>
+      </c>
+      <c r="B270" s="117" t="inlineStr">
+        <is>
+          <t>Veneer thickness 1.0 mm</t>
+        </is>
+      </c>
+      <c r="C270" s="129" t="n">
+        <v>1</v>
+      </c>
+      <c r="D270" s="113" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E270" s="113" t="inlineStr">
+        <is>
+          <t>Industry sliced thickness</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="113" t="inlineStr">
+        <is>
+          <t>VEN_T_12</t>
+        </is>
+      </c>
+      <c r="B271" s="117" t="inlineStr">
+        <is>
+          <t>Veneer thickness 1.2 mm</t>
+        </is>
+      </c>
+      <c r="C271" s="129" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="D271" s="113" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E271" s="113" t="inlineStr">
+        <is>
+          <t>Industry sliced thickness</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="113" t="inlineStr">
+        <is>
+          <t>VEN_M2_06</t>
+        </is>
+      </c>
+      <c r="B272" s="117" t="inlineStr">
+        <is>
+          <t>Veneer cost per m2 usable, 0.6 mm (wood + slicing fee)</t>
+        </is>
+      </c>
+      <c r="C272" s="129">
+        <f>C263*C269/1000/C267+C268</f>
+        <v/>
+      </c>
+      <c r="D272" s="113" t="inlineStr">
+        <is>
+          <t>IDR/m²</t>
+        </is>
+      </c>
+      <c r="E272" s="113" t="inlineStr">
+        <is>
+          <t>Formula: log price x thickness / effective yield + fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="113" t="inlineStr">
+        <is>
+          <t>VEN_M2_10</t>
+        </is>
+      </c>
+      <c r="B273" s="117" t="inlineStr">
+        <is>
+          <t>Veneer cost per m2 usable, 1.0 mm (wood + slicing fee)</t>
+        </is>
+      </c>
+      <c r="C273" s="129">
+        <f>C263*C270/1000/C267+C268</f>
+        <v/>
+      </c>
+      <c r="D273" s="113" t="inlineStr">
+        <is>
+          <t>IDR/m²</t>
+        </is>
+      </c>
+      <c r="E273" s="113" t="inlineStr">
+        <is>
+          <t>Formula: log price x thickness / effective yield + fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="113" t="inlineStr">
+        <is>
+          <t>VEN_M2_12</t>
+        </is>
+      </c>
+      <c r="B274" s="117" t="inlineStr">
+        <is>
+          <t>Veneer cost per m2 usable, 1.2 mm (wood + slicing fee)</t>
+        </is>
+      </c>
+      <c r="C274" s="129">
+        <f>C263*C271/1000/C267+C268</f>
+        <v/>
+      </c>
+      <c r="D274" s="113" t="inlineStr">
+        <is>
+          <t>IDR/m²</t>
+        </is>
+      </c>
+      <c r="E274" s="113" t="inlineStr">
+        <is>
+          <t>Formula: log price x thickness / effective yield + fee</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="113" t="inlineStr">
+        <is>
+          <t>VEN_FACE_06</t>
+        </is>
+      </c>
+      <c r="B275" s="117" t="inlineStr">
+        <is>
+          <t>Veneer added per board face, 0.6 mm (veneer + glue/tape on a full sheet + pressing labour)</t>
+        </is>
+      </c>
+      <c r="C275" s="129">
+        <f>(C272+$C$28)*(LISTS!$F$6*LISTS!$F$7/1000000)+$C$32</f>
+        <v/>
+      </c>
+      <c r="D275" s="113" t="inlineStr">
+        <is>
+          <t>IDR/face</t>
+        </is>
+      </c>
+      <c r="E275" s="113" t="inlineStr">
+        <is>
+          <t>Formula: (veneer m2 + glue_tape) x sheet area + ven_labour</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="113" t="inlineStr">
+        <is>
+          <t>VEN_FACE_10</t>
+        </is>
+      </c>
+      <c r="B276" s="117" t="inlineStr">
+        <is>
+          <t>Veneer added per board face, 1.0 mm (veneer + glue/tape on a full sheet + pressing labour)</t>
+        </is>
+      </c>
+      <c r="C276" s="129">
+        <f>(C273+$C$28)*(LISTS!$F$6*LISTS!$F$7/1000000)+$C$32</f>
+        <v/>
+      </c>
+      <c r="D276" s="113" t="inlineStr">
+        <is>
+          <t>IDR/face</t>
+        </is>
+      </c>
+      <c r="E276" s="113" t="inlineStr">
+        <is>
+          <t>Formula: (veneer m2 + glue_tape) x sheet area + ven_labour</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="113" t="inlineStr">
+        <is>
+          <t>VEN_FACE_12</t>
+        </is>
+      </c>
+      <c r="B277" s="117" t="inlineStr">
+        <is>
+          <t>Veneer added per board face, 1.2 mm (veneer + glue/tape on a full sheet + pressing labour)</t>
+        </is>
+      </c>
+      <c r="C277" s="129">
+        <f>(C274+$C$28)*(LISTS!$F$6*LISTS!$F$7/1000000)+$C$32</f>
+        <v/>
+      </c>
+      <c r="D277" s="113" t="inlineStr">
+        <is>
+          <t>IDR/face</t>
+        </is>
+      </c>
+      <c r="E277" s="113" t="inlineStr">
+        <is>
+          <t>Formula: (veneer m2 + glue_tape) x sheet area + ven_labour</t>
+        </is>
+      </c>
+    </row>
+    <row r="278"/>
+    <row r="279">
+      <c r="A279" s="127" t="inlineStr">
+        <is>
+          <t>VENEERED BOARDS 1.0 / 1.2 mm (code + -V10 or -V12). Equals the default board code + number of faces x (face cost of that thickness - 0.6 mm face).</t>
+        </is>
+      </c>
+      <c r="B279" s="98" t="n"/>
+      <c r="C279" s="98" t="n"/>
+      <c r="D279" s="98" t="n"/>
+      <c r="E279" s="98" t="n"/>
+      <c r="F279" s="98" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B280" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 18 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C280" s="128">
+        <f>C232+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D280" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E280" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F280" s="95" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B281" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 18 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C281" s="128">
+        <f>C232+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D281" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E281" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F281" s="95" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B282" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 18 mm, Mindi double face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C282" s="128">
+        <f>C233+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D282" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E282" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F282" s="95" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B283" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 18 mm, Mindi double face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C283" s="128">
+        <f>C233+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D283" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E283" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F283" s="95" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B284" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 15 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C284" s="128">
+        <f>C234+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D284" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E284" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F284" s="95" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B285" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 15 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C285" s="128">
+        <f>C234+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D285" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E285" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F285" s="95" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B286" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 15 mm, Mindi double face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C286" s="128">
+        <f>C235+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D286" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E286" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F286" s="95" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B287" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 15 mm, Mindi double face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C287" s="128">
+        <f>C235+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D287" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E287" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F287" s="95" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B288" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 12 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C288" s="128">
+        <f>C236+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D288" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E288" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F288" s="95" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B289" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 12 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C289" s="128">
+        <f>C236+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D289" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E289" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F289" s="95" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B290" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 12 mm, Mindi double face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C290" s="128">
+        <f>C237+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D290" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E290" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F290" s="95" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B291" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 12 mm, Mindi double face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C291" s="128">
+        <f>C237+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D291" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E291" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F291" s="95" t="n"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B292" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 9 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C292" s="128">
+        <f>C238+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D292" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E292" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F292" s="95" t="n"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B293" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 9 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C293" s="128">
+        <f>C238+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D293" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E293" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F293" s="95" t="n"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B294" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 9 mm, Mindi double face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C294" s="128">
+        <f>C239+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D294" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E294" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F294" s="95" t="n"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B295" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 9 mm, Mindi double face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C295" s="128">
+        <f>C239+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D295" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E295" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F295" s="95" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B296" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 6 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C296" s="128">
+        <f>C240+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D296" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E296" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F296" s="95" t="n"/>
+    </row>
+    <row r="297">
+      <c r="A297" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B297" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 6 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C297" s="128">
+        <f>C240+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D297" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E297" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F297" s="95" t="n"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B298" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 6 mm, Mindi double face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C298" s="128">
+        <f>C241+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D298" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E298" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F298" s="95" t="n"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B299" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 6 mm, Mindi double face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C299" s="128">
+        <f>C241+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D299" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E299" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F299" s="95" t="n"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B300" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 3 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C300" s="128">
+        <f>C242+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D300" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E300" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F300" s="95" t="n"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B301" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 3 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C301" s="128">
+        <f>C242+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D301" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E301" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F301" s="95" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B302" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 3 mm, Mindi double face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C302" s="128">
+        <f>C243+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D302" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E302" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F302" s="95" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B303" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E2 3 mm, Mindi double face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C303" s="128">
+        <f>C243+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D303" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E303" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F303" s="95" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B304" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 18 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C304" s="128">
+        <f>C244+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D304" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E304" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F304" s="95" t="n"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B305" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 18 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C305" s="128">
+        <f>C244+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D305" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E305" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F305" s="95" t="n"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B306" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 18 mm, Mindi double face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C306" s="128">
+        <f>C245+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D306" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E306" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F306" s="95" t="n"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B307" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 18 mm, Mindi double face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C307" s="128">
+        <f>C245+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D307" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E307" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F307" s="95" t="n"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-15-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B308" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 15 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C308" s="128">
+        <f>C246+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D308" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E308" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F308" s="95" t="n"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-15-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B309" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 15 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C309" s="128">
+        <f>C246+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D309" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E309" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F309" s="95" t="n"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-12-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B310" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 12 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C310" s="128">
+        <f>C247+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D310" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E310" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F310" s="95" t="n"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-12-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B311" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 12 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C311" s="128">
+        <f>C247+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D311" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E311" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F311" s="95" t="n"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-9-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B312" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 9 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C312" s="128">
+        <f>C248+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D312" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E312" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F312" s="95" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-9-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B313" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 9 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C313" s="128">
+        <f>C248+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D313" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E313" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F313" s="95" t="n"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-6-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B314" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 6 mm, Mindi single face (1.0 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C314" s="128">
+        <f>C249+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D314" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E314" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F314" s="95" t="n"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-6-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B315" s="93" t="inlineStr">
+        <is>
+          <t>MDF E2 6 mm, Mindi single face (1.2 mm veneer)</t>
+        </is>
+      </c>
+      <c r="C315" s="128">
+        <f>C249+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D315" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E315" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F315" s="95" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5:C400">
@@ -17476,7 +18858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="16" customWidth="1" style="59" min="1" max="2"/>
@@ -17864,51 +19246,257 @@
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="59">
-      <c r="B33" s="2" t="n"/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MSF-V10</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="59">
-      <c r="B34" s="2" t="n"/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MSF-V12</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="59">
-      <c r="B35" s="2" t="n"/>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MDF-V10</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="59">
-      <c r="B36" s="2" t="n"/>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-18-MDF-V12</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="59">
-      <c r="B37" s="2" t="n"/>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" s="59"/>
-    <row r="39" ht="15.75" customHeight="1" s="59"/>
-    <row r="40" ht="15.75" customHeight="1" s="59"/>
-    <row r="41" ht="15.75" customHeight="1" s="59"/>
-    <row r="42" ht="15.75" customHeight="1" s="59"/>
-    <row r="43" ht="15.75" customHeight="1" s="59"/>
-    <row r="44" ht="15.75" customHeight="1" s="59"/>
-    <row r="45" ht="15.75" customHeight="1" s="59"/>
-    <row r="46" ht="15.75" customHeight="1" s="59"/>
-    <row r="47" ht="15.75" customHeight="1" s="59"/>
-    <row r="48" ht="15.75" customHeight="1" s="59"/>
-    <row r="49" ht="15.75" customHeight="1" s="59"/>
-    <row r="50" ht="15.75" customHeight="1" s="59"/>
-    <row r="51" ht="15.75" customHeight="1" s="59"/>
-    <row r="52" ht="15.75" customHeight="1" s="59"/>
-    <row r="53" ht="15.75" customHeight="1" s="59"/>
-    <row r="54" ht="15.75" customHeight="1" s="59"/>
-    <row r="55" ht="15.75" customHeight="1" s="59"/>
-    <row r="56" ht="15.75" customHeight="1" s="59"/>
-    <row r="57" ht="15.75" customHeight="1" s="59"/>
-    <row r="58" ht="15.75" customHeight="1" s="59"/>
-    <row r="59" ht="15.75" customHeight="1" s="59"/>
-    <row r="60" ht="15.75" customHeight="1" s="59"/>
-    <row r="61" ht="15.75" customHeight="1" s="59"/>
-    <row r="62" ht="15.75" customHeight="1" s="59"/>
-    <row r="63" ht="15.75" customHeight="1" s="59"/>
-    <row r="64" ht="15.75" customHeight="1" s="59"/>
-    <row r="65" ht="15.75" customHeight="1" s="59"/>
-    <row r="66" ht="15.75" customHeight="1" s="59"/>
-    <row r="67" ht="15.75" customHeight="1" s="59"/>
-    <row r="68" ht="15.75" customHeight="1" s="59"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1" s="59">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="59">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" s="59">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-15-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="59">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="59">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="59">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="59">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-12-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="59">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1" s="59">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="59">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1" s="59">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-9-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1" s="59">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="59">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="59">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1" s="59">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-6-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="59">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1" s="59">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1" s="59">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1" s="59">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>LND-PLY-E2-3-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1" s="59">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15.75" customHeight="1" s="59">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customHeight="1" s="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1" s="59">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-18-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1" s="59">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-15-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1" s="59">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-15-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15.75" customHeight="1" s="59">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-12-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15.75" customHeight="1" s="59">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-12-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="15.75" customHeight="1" s="59">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-9-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="15.75" customHeight="1" s="59">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-9-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15.75" customHeight="1" s="59">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-6-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="15.75" customHeight="1" s="59">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>LND-MDF-E2-6-MSF-V12</t>
+        </is>
+      </c>
+    </row>
     <row r="69" ht="15.75" customHeight="1" s="59"/>
     <row r="70" ht="15.75" customHeight="1" s="59"/>
     <row r="71" ht="15.75" customHeight="1" s="59"/>

</xml_diff>

<commit_message>
feat(rules): ALL plywood and MDF use grade E0 (meeting 19 Oct 2026) - replaces E2 lock; E0 veneered boards in RATES; to_e0 normaliser; config rebuilt on E0; specs converted; tests
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -10239,7 +10239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I315"/>
+  <dimension ref="A1:I389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="59" min="1" max="1"/>
@@ -14763,12 +14763,12 @@
       </c>
       <c r="B174" s="117" t="inlineStr">
         <is>
-          <t>Board grade for ALL plywood and MDF (LOCKED E2, rule 19 Oct 2026). Do not change.</t>
+          <t>Board grade for ALL plywood and MDF (LOCKED E0, meeting rule 19 Oct 2026). Replaces E2.</t>
         </is>
       </c>
       <c r="C174" s="118" t="inlineStr">
         <is>
-          <t>E2</t>
+          <t>E0</t>
         </is>
       </c>
       <c r="D174" s="113" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="E174" s="113" t="inlineStr">
         <is>
-          <t>Rule: plywood (B group) and MDF (C group) always E2, landed Kudus. E0 / CARB rows are reference only.</t>
+          <t>Rule: plywood and MDF always E0, landed Kudus. E2 / CARB rows are reference only.</t>
         </is>
       </c>
       <c r="F174" s="95" t="n"/>
@@ -18841,6 +18841,1963 @@
         </is>
       </c>
       <c r="F315" s="95" t="n"/>
+    </row>
+    <row r="316"/>
+    <row r="317">
+      <c r="A317" s="127" t="inlineStr">
+        <is>
+          <t>E0 BOARDS (rule 19 Oct 2026, meeting): ALL plywood and MDF use grade E0. Veneered E0 boards = raw E0 landed board + faces x veneer face cost (0.6 mm default; -V10 / -V12 for 1.0 / 1.2 mm).</t>
+        </is>
+      </c>
+      <c r="B317" s="98" t="n"/>
+      <c r="C317" s="98" t="n"/>
+      <c r="D317" s="98" t="n"/>
+      <c r="E317" s="98" t="n"/>
+      <c r="F317" s="98" t="n"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-3-MSF</t>
+        </is>
+      </c>
+      <c r="B318" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 3 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C318" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-3",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D318" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E318" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F318" s="95" t="n"/>
+    </row>
+    <row r="319">
+      <c r="A319" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-3-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B319" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 3 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C319" s="128">
+        <f>C318+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D319" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E319" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F319" s="95" t="n"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-3-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B320" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 3 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C320" s="128">
+        <f>C318+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D320" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E320" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F320" s="95" t="n"/>
+    </row>
+    <row r="321">
+      <c r="A321" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-3-MDF</t>
+        </is>
+      </c>
+      <c r="B321" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 3 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C321" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-3",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D321" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E321" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F321" s="95" t="n"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-3-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B322" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 3 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C322" s="128">
+        <f>C321+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D322" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E322" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F322" s="95" t="n"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-3-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B323" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 3 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C323" s="128">
+        <f>C321+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D323" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E323" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F323" s="95" t="n"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-6-MSF</t>
+        </is>
+      </c>
+      <c r="B324" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 6 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C324" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-6",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D324" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E324" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F324" s="95" t="n"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-6-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B325" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 6 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C325" s="128">
+        <f>C324+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D325" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E325" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F325" s="95" t="n"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-6-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B326" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 6 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C326" s="128">
+        <f>C324+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D326" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E326" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F326" s="95" t="n"/>
+    </row>
+    <row r="327">
+      <c r="A327" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-6-MDF</t>
+        </is>
+      </c>
+      <c r="B327" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 6 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C327" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-6",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D327" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E327" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F327" s="95" t="n"/>
+    </row>
+    <row r="328">
+      <c r="A328" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-6-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B328" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 6 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C328" s="128">
+        <f>C327+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D328" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E328" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F328" s="95" t="n"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-6-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B329" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 6 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C329" s="128">
+        <f>C327+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D329" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E329" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F329" s="95" t="n"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-9-MSF</t>
+        </is>
+      </c>
+      <c r="B330" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 9 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C330" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-9",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D330" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E330" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F330" s="95" t="n"/>
+    </row>
+    <row r="331">
+      <c r="A331" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-9-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B331" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 9 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C331" s="128">
+        <f>C330+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D331" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E331" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F331" s="95" t="n"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-9-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B332" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 9 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C332" s="128">
+        <f>C330+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D332" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E332" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F332" s="95" t="n"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-9-MDF</t>
+        </is>
+      </c>
+      <c r="B333" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 9 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C333" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-9",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D333" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E333" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F333" s="95" t="n"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-9-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B334" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 9 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C334" s="128">
+        <f>C333+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D334" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E334" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F334" s="95" t="n"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-9-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B335" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 9 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C335" s="128">
+        <f>C333+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D335" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E335" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F335" s="95" t="n"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-12-MSF</t>
+        </is>
+      </c>
+      <c r="B336" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 12 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C336" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-12",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D336" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E336" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F336" s="95" t="n"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-12-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B337" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 12 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C337" s="128">
+        <f>C336+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D337" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E337" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F337" s="95" t="n"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-12-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B338" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 12 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C338" s="128">
+        <f>C336+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D338" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E338" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F338" s="95" t="n"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-12-MDF</t>
+        </is>
+      </c>
+      <c r="B339" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 12 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C339" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-12",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D339" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E339" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F339" s="95" t="n"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-12-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B340" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 12 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C340" s="128">
+        <f>C339+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D340" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E340" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F340" s="95" t="n"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-12-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B341" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 12 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C341" s="128">
+        <f>C339+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D341" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E341" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F341" s="95" t="n"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-15-MSF</t>
+        </is>
+      </c>
+      <c r="B342" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 15 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C342" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-15",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D342" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E342" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F342" s="95" t="n"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-15-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B343" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 15 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C343" s="128">
+        <f>C342+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D343" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E343" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F343" s="95" t="n"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-15-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B344" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 15 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C344" s="128">
+        <f>C342+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D344" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E344" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F344" s="95" t="n"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-15-MDF</t>
+        </is>
+      </c>
+      <c r="B345" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 15 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C345" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-15",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D345" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E345" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F345" s="95" t="n"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-15-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B346" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 15 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C346" s="128">
+        <f>C345+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D346" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E346" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F346" s="95" t="n"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-15-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B347" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 15 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C347" s="128">
+        <f>C345+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D347" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E347" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F347" s="95" t="n"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-18-MSF</t>
+        </is>
+      </c>
+      <c r="B348" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 18 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C348" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-18",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D348" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E348" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F348" s="95" t="n"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-18-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B349" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 18 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C349" s="128">
+        <f>C348+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D349" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E349" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F349" s="95" t="n"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-18-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B350" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 18 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C350" s="128">
+        <f>C348+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D350" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E350" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F350" s="95" t="n"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-18-MDF</t>
+        </is>
+      </c>
+      <c r="B351" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 18 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C351" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-PLY-E0-18",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D351" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E351" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F351" s="95" t="n"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-18-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B352" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 18 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C352" s="128">
+        <f>C351+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D352" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E352" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F352" s="95" t="n"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="95" t="inlineStr">
+        <is>
+          <t>LND-PLY-E0-18-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B353" s="93" t="inlineStr">
+        <is>
+          <t>Plywood E0 18 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C353" s="128">
+        <f>C351+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D353" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E353" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F353" s="95" t="n"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-3-MSF</t>
+        </is>
+      </c>
+      <c r="B354" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 3 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C354" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-3",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D354" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E354" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F354" s="95" t="n"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-3-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B355" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 3 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C355" s="128">
+        <f>C354+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D355" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E355" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F355" s="95" t="n"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-3-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B356" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 3 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C356" s="128">
+        <f>C354+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D356" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E356" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F356" s="95" t="n"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-3-MDF</t>
+        </is>
+      </c>
+      <c r="B357" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 3 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C357" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-3",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D357" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E357" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F357" s="95" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-3-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B358" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 3 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C358" s="128">
+        <f>C357+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D358" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E358" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F358" s="95" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-3-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B359" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 3 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C359" s="128">
+        <f>C357+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D359" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E359" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F359" s="95" t="n"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-6-MSF</t>
+        </is>
+      </c>
+      <c r="B360" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 6 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C360" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-6",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D360" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E360" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F360" s="95" t="n"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-6-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B361" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 6 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C361" s="128">
+        <f>C360+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D361" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E361" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F361" s="95" t="n"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-6-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B362" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 6 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C362" s="128">
+        <f>C360+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D362" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E362" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F362" s="95" t="n"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-6-MDF</t>
+        </is>
+      </c>
+      <c r="B363" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 6 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C363" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-6",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D363" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E363" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F363" s="95" t="n"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-6-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B364" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 6 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C364" s="128">
+        <f>C363+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D364" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E364" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F364" s="95" t="n"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-6-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B365" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 6 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C365" s="128">
+        <f>C363+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D365" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E365" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F365" s="95" t="n"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-9-MSF</t>
+        </is>
+      </c>
+      <c r="B366" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 9 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C366" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-9",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D366" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E366" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F366" s="95" t="n"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-9-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B367" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 9 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C367" s="128">
+        <f>C366+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D367" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E367" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F367" s="95" t="n"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-9-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B368" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 9 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C368" s="128">
+        <f>C366+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D368" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E368" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F368" s="95" t="n"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-9-MDF</t>
+        </is>
+      </c>
+      <c r="B369" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 9 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C369" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-9",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D369" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E369" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F369" s="95" t="n"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-9-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B370" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 9 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C370" s="128">
+        <f>C369+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D370" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E370" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F370" s="95" t="n"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-9-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B371" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 9 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C371" s="128">
+        <f>C369+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D371" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E371" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F371" s="95" t="n"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MSF</t>
+        </is>
+      </c>
+      <c r="B372" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 12 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C372" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-12",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D372" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E372" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F372" s="95" t="n"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B373" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 12 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C373" s="128">
+        <f>C372+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D373" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E373" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F373" s="95" t="n"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B374" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 12 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C374" s="128">
+        <f>C372+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D374" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E374" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F374" s="95" t="n"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MDF</t>
+        </is>
+      </c>
+      <c r="B375" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 12 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C375" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-12",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D375" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E375" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F375" s="95" t="n"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B376" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 12 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C376" s="128">
+        <f>C375+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D376" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E376" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F376" s="95" t="n"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B377" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 12 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C377" s="128">
+        <f>C375+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D377" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E377" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F377" s="95" t="n"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MSF</t>
+        </is>
+      </c>
+      <c r="B378" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 15 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C378" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-15",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D378" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E378" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F378" s="95" t="n"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B379" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 15 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C379" s="128">
+        <f>C378+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D379" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E379" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F379" s="95" t="n"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B380" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 15 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C380" s="128">
+        <f>C378+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D380" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E380" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F380" s="95" t="n"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MDF</t>
+        </is>
+      </c>
+      <c r="B381" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 15 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C381" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-15",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D381" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E381" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F381" s="95" t="n"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B382" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 15 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C382" s="128">
+        <f>C381+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D382" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E382" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F382" s="95" t="n"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B383" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 15 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C383" s="128">
+        <f>C381+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D383" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E383" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F383" s="95" t="n"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MSF</t>
+        </is>
+      </c>
+      <c r="B384" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 18 mm, Mindi single face</t>
+        </is>
+      </c>
+      <c r="C384" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-18",$A$178:$A$215,0))+1*$C$175</f>
+        <v/>
+      </c>
+      <c r="D384" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E384" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F384" s="95" t="n"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MSF-V10</t>
+        </is>
+      </c>
+      <c r="B385" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 18 mm, Mindi single face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C385" s="128">
+        <f>C384+1*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D385" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E385" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F385" s="95" t="n"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MSF-V12</t>
+        </is>
+      </c>
+      <c r="B386" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 18 mm, Mindi single face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C386" s="128">
+        <f>C384+1*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D386" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E386" s="95" t="inlineStr">
+        <is>
+          <t>1 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F386" s="95" t="n"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MDF</t>
+        </is>
+      </c>
+      <c r="B387" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 18 mm, Mindi double face</t>
+        </is>
+      </c>
+      <c r="C387" s="128">
+        <f>INDEX($C$178:$C$215,MATCH("LND-MDF-E0-18",$A$178:$A$215,0))+2*$C$175</f>
+        <v/>
+      </c>
+      <c r="D387" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E387" s="95" t="inlineStr">
+        <is>
+          <t>E0 raw landed + veneer face (0.6 mm)</t>
+        </is>
+      </c>
+      <c r="F387" s="95" t="n"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MDF-V10</t>
+        </is>
+      </c>
+      <c r="B388" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 18 mm, Mindi double face, 1.0 mm veneer</t>
+        </is>
+      </c>
+      <c r="C388" s="128">
+        <f>C387+2*(C276-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D388" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E388" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.0 mm</t>
+        </is>
+      </c>
+      <c r="F388" s="95" t="n"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="95" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MDF-V12</t>
+        </is>
+      </c>
+      <c r="B389" s="93" t="inlineStr">
+        <is>
+          <t>MDF E0 18 mm, Mindi double face, 1.2 mm veneer</t>
+        </is>
+      </c>
+      <c r="C389" s="128">
+        <f>C387+2*(C277-$C$175)</f>
+        <v/>
+      </c>
+      <c r="D389" s="95" t="inlineStr">
+        <is>
+          <t>IDR/sheet</t>
+        </is>
+      </c>
+      <c r="E389" s="95" t="inlineStr">
+        <is>
+          <t>2 face(s) at 1.2 mm</t>
+        </is>
+      </c>
+      <c r="F389" s="95" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5:C400">
@@ -18858,7 +20815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="16" customWidth="1" style="59" min="1" max="2"/>
@@ -18916,7 +20873,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-3</t>
+          <t>LND-PLY-E0-3</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -18946,7 +20903,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-6</t>
+          <t>LND-PLY-E0-6</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -18976,7 +20933,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-9</t>
+          <t>LND-PLY-E0-9</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -19001,7 +20958,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-12</t>
+          <t>LND-PLY-E0-12</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -19021,7 +20978,7 @@
     <row r="7">
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-15</t>
+          <t>LND-PLY-E0-15</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -19041,7 +20998,7 @@
     <row r="8">
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-18</t>
+          <t>LND-PLY-E0-18</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -19056,7 +21013,7 @@
     <row r="9">
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-3</t>
+          <t>LND-MDF-E0-3</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -19071,7 +21028,7 @@
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-6</t>
+          <t>LND-MDF-E0-6</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -19086,7 +21043,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-9</t>
+          <t>LND-MDF-E0-9</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -19101,420 +21058,528 @@
     <row r="12">
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-12</t>
+          <t>LND-MDF-E0-12</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-15</t>
+          <t>LND-MDF-E0-15</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-18</t>
+          <t>LND-MDF-E0-18</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-18-MSF</t>
+          <t>LND-PLY-E0-3-MSF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-18-MDF</t>
+          <t>LND-PLY-E0-3-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-15-MSF</t>
+          <t>LND-PLY-E0-3-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-15-MDF</t>
+          <t>LND-PLY-E0-3-MDF</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-12-MSF</t>
+          <t>LND-PLY-E0-3-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-12-MDF</t>
+          <t>LND-PLY-E0-3-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="59">
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-9-MSF</t>
+          <t>LND-PLY-E0-6-MSF</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="59">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-9-MDF</t>
+          <t>LND-PLY-E0-6-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="59">
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-6-MSF</t>
+          <t>LND-PLY-E0-6-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="59">
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-6-MDF</t>
+          <t>LND-PLY-E0-6-MDF</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="59">
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-3-MSF</t>
+          <t>LND-PLY-E0-6-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="59">
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-3-MDF</t>
+          <t>LND-PLY-E0-6-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="59">
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-18-MSF</t>
+          <t>LND-PLY-E0-9-MSF</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="59">
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-18-MDF</t>
+          <t>LND-PLY-E0-9-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="59">
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-15-MSF</t>
+          <t>LND-PLY-E0-9-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="59">
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-12-MSF</t>
+          <t>LND-PLY-E0-9-MDF</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="59">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-9-MSF</t>
+          <t>LND-PLY-E0-9-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="59">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-6-MSF</t>
+          <t>LND-PLY-E0-9-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="59">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-18-MSF-V10</t>
+          <t>LND-PLY-E0-12-MSF</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="59">
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-18-MSF-V12</t>
+          <t>LND-PLY-E0-12-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="59">
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-18-MDF-V10</t>
+          <t>LND-PLY-E0-12-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="59">
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-18-MDF-V12</t>
+          <t>LND-PLY-E0-12-MDF</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="59">
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-15-MSF-V10</t>
+          <t>LND-PLY-E0-12-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="59">
       <c r="B38" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-15-MSF-V12</t>
+          <t>LND-PLY-E0-12-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="59">
       <c r="B39" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-15-MDF-V10</t>
+          <t>LND-PLY-E0-15-MSF</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="59">
       <c r="B40" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-15-MDF-V12</t>
+          <t>LND-PLY-E0-15-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="59">
       <c r="B41" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-12-MSF-V10</t>
+          <t>LND-PLY-E0-15-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="59">
       <c r="B42" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-12-MSF-V12</t>
+          <t>LND-PLY-E0-15-MDF</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="59">
       <c r="B43" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-12-MDF-V10</t>
+          <t>LND-PLY-E0-15-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="59">
       <c r="B44" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-12-MDF-V12</t>
+          <t>LND-PLY-E0-15-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="59">
       <c r="B45" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-9-MSF-V10</t>
+          <t>LND-PLY-E0-18-MSF</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="59">
       <c r="B46" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-9-MSF-V12</t>
+          <t>LND-PLY-E0-18-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="59">
       <c r="B47" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-9-MDF-V10</t>
+          <t>LND-PLY-E0-18-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="59">
       <c r="B48" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-9-MDF-V12</t>
+          <t>LND-PLY-E0-18-MDF</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="59">
       <c r="B49" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-6-MSF-V10</t>
+          <t>LND-PLY-E0-18-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="59">
       <c r="B50" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-6-MSF-V12</t>
+          <t>LND-PLY-E0-18-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="59">
       <c r="B51" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-6-MDF-V10</t>
+          <t>LND-MDF-E0-3-MSF</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="59">
       <c r="B52" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-6-MDF-V12</t>
+          <t>LND-MDF-E0-3-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="59">
       <c r="B53" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-3-MSF-V10</t>
+          <t>LND-MDF-E0-3-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="59">
       <c r="B54" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-3-MSF-V12</t>
+          <t>LND-MDF-E0-3-MDF</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="59">
       <c r="B55" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-3-MDF-V10</t>
+          <t>LND-MDF-E0-3-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="59">
       <c r="B56" t="inlineStr">
         <is>
-          <t>LND-PLY-E2-3-MDF-V12</t>
+          <t>LND-MDF-E0-3-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="59">
       <c r="B57" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-18-MSF-V10</t>
+          <t>LND-MDF-E0-6-MSF</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="59">
       <c r="B58" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-18-MSF-V12</t>
+          <t>LND-MDF-E0-6-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-18-MDF-V10</t>
+          <t>LND-MDF-E0-6-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="59">
       <c r="B60" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-18-MDF-V12</t>
+          <t>LND-MDF-E0-6-MDF</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="59">
       <c r="B61" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-15-MSF-V10</t>
+          <t>LND-MDF-E0-6-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="59">
       <c r="B62" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-15-MSF-V12</t>
+          <t>LND-MDF-E0-6-MDF-V12</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="59">
       <c r="B63" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-12-MSF-V10</t>
+          <t>LND-MDF-E0-9-MSF</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="59">
       <c r="B64" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-12-MSF-V12</t>
+          <t>LND-MDF-E0-9-MSF-V10</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="59">
       <c r="B65" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-9-MSF-V10</t>
+          <t>LND-MDF-E0-9-MSF-V12</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="59">
       <c r="B66" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-9-MSF-V12</t>
+          <t>LND-MDF-E0-9-MDF</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="59">
       <c r="B67" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-6-MSF-V10</t>
+          <t>LND-MDF-E0-9-MDF-V10</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="59">
       <c r="B68" t="inlineStr">
         <is>
-          <t>LND-MDF-E2-6-MSF-V12</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="15.75" customHeight="1" s="59"/>
-    <row r="70" ht="15.75" customHeight="1" s="59"/>
-    <row r="71" ht="15.75" customHeight="1" s="59"/>
-    <row r="72" ht="15.75" customHeight="1" s="59"/>
-    <row r="73" ht="15.75" customHeight="1" s="59"/>
-    <row r="74" ht="15.75" customHeight="1" s="59"/>
-    <row r="75" ht="15.75" customHeight="1" s="59"/>
-    <row r="76" ht="15.75" customHeight="1" s="59"/>
-    <row r="77" ht="15.75" customHeight="1" s="59"/>
-    <row r="78" ht="15.75" customHeight="1" s="59"/>
-    <row r="79" ht="15.75" customHeight="1" s="59"/>
-    <row r="80" ht="15.75" customHeight="1" s="59"/>
-    <row r="81" ht="15.75" customHeight="1" s="59"/>
-    <row r="82" ht="15.75" customHeight="1" s="59"/>
-    <row r="83" ht="15.75" customHeight="1" s="59"/>
-    <row r="84" ht="15.75" customHeight="1" s="59"/>
-    <row r="85" ht="15.75" customHeight="1" s="59"/>
-    <row r="86" ht="15.75" customHeight="1" s="59"/>
+          <t>LND-MDF-E0-9-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15.75" customHeight="1" s="59">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="15.75" customHeight="1" s="59">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="15.75" customHeight="1" s="59">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="15.75" customHeight="1" s="59">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="15.75" customHeight="1" s="59">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="15.75" customHeight="1" s="59">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-12-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="15.75" customHeight="1" s="59">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="15.75" customHeight="1" s="59">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="15.75" customHeight="1" s="59">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="15.75" customHeight="1" s="59">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="15.75" customHeight="1" s="59">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="15.75" customHeight="1" s="59">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-15-MDF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="15.75" customHeight="1" s="59">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15.75" customHeight="1" s="59">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MSF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15.75" customHeight="1" s="59">
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MSF-V12</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15.75" customHeight="1" s="59">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15.75" customHeight="1" s="59">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MDF-V10</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15.75" customHeight="1" s="59">
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>LND-MDF-E0-18-MDF-V12</t>
+        </is>
+      </c>
+    </row>
     <row r="87" ht="15.75" customHeight="1" s="59"/>
     <row r="88" ht="15.75" customHeight="1" s="59"/>
     <row r="89" ht="15.75" customHeight="1" s="59"/>

</xml_diff>

<commit_message>
feat(metal): METAL parts priced as hollow steel (length x IDR/m from the supplier list, wall via RATES!HOLLOW_WALL=1.2); sheet formula follows RATES; config loads prices; tests
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -14643,6 +14643,7 @@
       <c r="H168" s="95" t="n"/>
       <c r="I168" s="95" t="n"/>
     </row>
+    <row r="169"/>
     <row r="170">
       <c r="A170" s="97" t="inlineStr">
         <is>
@@ -14853,6 +14854,7 @@
       <c r="H176" s="95" t="n"/>
       <c r="I176" s="95" t="n"/>
     </row>
+    <row r="177"/>
     <row r="178">
       <c r="A178" s="119" t="inlineStr">
         <is>
@@ -16373,6 +16375,7 @@
         <v>933</v>
       </c>
     </row>
+    <row r="216"/>
     <row r="217">
       <c r="A217" s="97" t="inlineStr">
         <is>
@@ -16676,6 +16679,7 @@
       <c r="H225" s="95" t="n"/>
       <c r="I225" s="95" t="n"/>
     </row>
+    <row r="226"/>
     <row r="227">
       <c r="A227" s="97" t="inlineStr">
         <is>
@@ -16769,6 +16773,7 @@
       <c r="H229" s="95" t="n"/>
       <c r="I229" s="95" t="n"/>
     </row>
+    <row r="230"/>
     <row r="231">
       <c r="A231" s="127" t="inlineStr">
         <is>
@@ -17252,10 +17257,11 @@
       <c r="H249" s="95" t="n"/>
       <c r="I249" s="95" t="n"/>
     </row>
+    <row r="250"/>
     <row r="251">
       <c r="A251" s="127" t="inlineStr">
         <is>
-          <t>METAL (added 19 Oct 2026). Value EMPTY: price not yet received. Fill column C; METAL parts cost 0 until filled.</t>
+          <t>METAL = black hollow steel (rule 19 Oct 2026). METAL parts are priced from the STEEL HOLLOW SECTION list below: length x qty x IDR/m of HOLLOW-&lt;a&gt;x&lt;b&gt;x&lt;wall&gt;. Set the wall thickness here.</t>
         </is>
       </c>
       <c r="B251" s="98" t="n"/>
@@ -17270,23 +17276,25 @@
     <row r="252">
       <c r="A252" s="113" t="inlineStr">
         <is>
-          <t>METAL_A</t>
+          <t>HOLLOW_WALL</t>
         </is>
       </c>
       <c r="B252" s="117" t="inlineStr">
         <is>
-          <t>Metal tier A (exposed, long), per m³ of component</t>
-        </is>
-      </c>
-      <c r="C252" s="129" t="n"/>
+          <t>Wall thickness used for ALL METAL parts (not on drawings)</t>
+        </is>
+      </c>
+      <c r="C252" s="129" t="n">
+        <v>1.2</v>
+      </c>
       <c r="D252" s="113" t="inlineStr">
         <is>
-          <t>IDR/m³</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="E252" s="113" t="inlineStr">
         <is>
-          <t>EMPTY: waiting for price</t>
+          <t>CONFIRM with factory: 1.2 assumed. Used: 0.8, 1.0, 1.2, 1.5, 1.8, 2.0 (as listed)</t>
         </is>
       </c>
       <c r="F252" s="95" t="n"/>
@@ -17305,7 +17313,11 @@
           <t>Metal tier B</t>
         </is>
       </c>
-      <c r="C253" s="129" t="n"/>
+      <c r="C253" s="129" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="D253" s="113" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -17313,7 +17325,7 @@
       </c>
       <c r="E253" s="113" t="inlineStr">
         <is>
-          <t>EMPTY: waiting for price</t>
+          <t>Not used: METAL parts are priced from the HOLLOW-... list</t>
         </is>
       </c>
       <c r="F253" s="95" t="n"/>
@@ -17332,7 +17344,11 @@
           <t>Metal tier C</t>
         </is>
       </c>
-      <c r="C254" s="129" t="n"/>
+      <c r="C254" s="129" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="D254" s="113" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -17340,7 +17356,7 @@
       </c>
       <c r="E254" s="113" t="inlineStr">
         <is>
-          <t>EMPTY: waiting for price</t>
+          <t>Not used: METAL parts are priced from the HOLLOW-... list</t>
         </is>
       </c>
       <c r="F254" s="95" t="n"/>
@@ -17359,7 +17375,11 @@
           <t>Metal tier D</t>
         </is>
       </c>
-      <c r="C255" s="129" t="n"/>
+      <c r="C255" s="129" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="D255" s="113" t="inlineStr">
         <is>
           <t>IDR/m³</t>
@@ -17367,7 +17387,7 @@
       </c>
       <c r="E255" s="113" t="inlineStr">
         <is>
-          <t>EMPTY: waiting for price</t>
+          <t>Not used: METAL parts are priced from the HOLLOW-... list</t>
         </is>
       </c>
       <c r="F255" s="95" t="n"/>
@@ -17386,7 +17406,11 @@
           <t>Brass, per kg (reference)</t>
         </is>
       </c>
-      <c r="C256" s="129" t="n"/>
+      <c r="C256" s="129" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="D256" s="113" t="inlineStr">
         <is>
           <t>IDR/kg</t>
@@ -17394,7 +17418,7 @@
       </c>
       <c r="E256" s="113" t="inlineStr">
         <is>
-          <t>EMPTY: waiting for price</t>
+          <t>Not used: METAL parts are priced from the HOLLOW-... list</t>
         </is>
       </c>
       <c r="F256" s="95" t="n"/>
@@ -17413,7 +17437,11 @@
           <t>Steel / hollow section, per kg (reference)</t>
         </is>
       </c>
-      <c r="C257" s="129" t="n"/>
+      <c r="C257" s="129" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
       <c r="D257" s="113" t="inlineStr">
         <is>
           <t>IDR/kg</t>
@@ -17421,7 +17449,7 @@
       </c>
       <c r="E257" s="113" t="inlineStr">
         <is>
-          <t>EMPTY: waiting for price</t>
+          <t>Not used: METAL parts are priced from the HOLLOW-... list</t>
         </is>
       </c>
       <c r="F257" s="95" t="n"/>

</xml_diff>

<commit_message>
feat(metal): hollow wall 0.8 mm for all METAL parts (manual via RATES!HOLLOW_WALL); fall back to next listed wall when a section has none (50x50, 40x60); sheet formula follows; tests
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -17285,7 +17285,7 @@
         </is>
       </c>
       <c r="C252" s="129" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="D252" s="113" t="inlineStr">
         <is>
@@ -17294,7 +17294,7 @@
       </c>
       <c r="E252" s="113" t="inlineStr">
         <is>
-          <t>CONFIRM with factory: 1.2 assumed. Used: 0.8, 1.0, 1.2, 1.5, 1.8, 2.0 (as listed)</t>
+          <t>0.8 mm for now (decision 19 Oct 2026). Change by hand. If a section has no such wall in the list (50x50, 40x60 start at 1.0), the next listed wall is used.</t>
         </is>
       </c>
       <c r="F252" s="95" t="n"/>

</xml_diff>

<commit_message>
METAL hollow: own section (rows 33-42) priced per metre; hollow code selectable in MATERIAL; metal no longer counted as timber m3 for fasteners; template, generators, layout, tests (64 pass), README K
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -393,7 +393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -647,6 +647,13 @@
     <xf numFmtId="2" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6471,7 +6478,7 @@
         <v/>
       </c>
     </row>
-    <row r="16">
+    <row r="16" s="59">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>SOLID WOOD: one line per component, mm, qty per ONE item</t>
@@ -6578,7 +6585,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" s="59">
       <c r="A18" s="9" t="n">
         <v>1</v>
       </c>
@@ -7208,93 +7215,128 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1" s="59">
-      <c r="A33" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B33" s="10" t="n"/>
-      <c r="C33" s="48" t="n"/>
-      <c r="D33" s="10" t="n"/>
-      <c r="E33" s="10" t="n"/>
-      <c r="F33" s="10" t="n"/>
-      <c r="G33" s="10" t="n"/>
-      <c r="H33" s="10" t="n"/>
-      <c r="I33" s="10" t="n"/>
-      <c r="J33" s="10" t="n"/>
-      <c r="K33" s="10" t="n"/>
-      <c r="L33" s="10" t="n"/>
-      <c r="M33" s="25">
-        <f>IF(OR(E33="",F33="",G33=""),"",E33*F33*G33/1000000000*IF(H33="",1,H33))</f>
-        <v/>
-      </c>
-      <c r="N33" s="19">
-        <f>IF(OR(E33="",F33=""),"",E33*F33/1000000*IF(H33="",1,H33))</f>
-        <v/>
-      </c>
-      <c r="O33" s="14">
-        <f>IF(E33="","",IF(K33&lt;&gt;"",K33,IF(AND(E33*F33*G33/1000000000&lt;LISTS!$F$4,MAX(E33,F33,G33)&lt;LISTS!$F$5),"D",IF(I33="N","C",IF(J33="Y","A-CURVED",IF(AND(MEDIAN(E33,F33,G33)&lt;=LISTS!$F$10,MAX(E33,F33,G33)&lt;=LISTS!$F$11),"B",IF(MAX(E33,F33,G33)&gt;=LISTS!$F$3,"A","B")))))))</f>
-        <v/>
-      </c>
-      <c r="P33" s="14" t="n"/>
-      <c r="Q33" s="14" t="n"/>
-      <c r="R33" s="14">
-        <f>IF(E33="","",IF(B33="","material?",IF(OR(F33="",G33=""),"size?",IF(I33="","exposed Y/N?",IF(H33="","qty?",IF(B33="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S33" s="12">
-        <f t="array" ref="S33">IF(OR(O33="",M33=""),"",IF(B33="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B33&amp;"_"&amp;SUBSTITUTE(O33,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T33" s="12">
-        <f>IF(ISNUMBER(S33),M33*S33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1" s="59">
-      <c r="A34" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="48" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
-      <c r="H34" s="10" t="n"/>
-      <c r="I34" s="10" t="n"/>
-      <c r="J34" s="10" t="n"/>
-      <c r="K34" s="10" t="n"/>
-      <c r="L34" s="10" t="n"/>
-      <c r="M34" s="25">
-        <f>IF(OR(E34="",F34="",G34=""),"",E34*F34*G34/1000000000*IF(H34="",1,H34))</f>
-        <v/>
-      </c>
-      <c r="N34" s="19">
-        <f>IF(OR(E34="",F34=""),"",E34*F34/1000000*IF(H34="",1,H34))</f>
-        <v/>
-      </c>
-      <c r="O34" s="14">
-        <f>IF(E34="","",IF(K34&lt;&gt;"",K34,IF(AND(E34*F34*G34/1000000000&lt;LISTS!$F$4,MAX(E34,F34,G34)&lt;LISTS!$F$5),"D",IF(I34="N","C",IF(J34="Y","A-CURVED",IF(AND(MEDIAN(E34,F34,G34)&lt;=LISTS!$F$10,MAX(E34,F34,G34)&lt;=LISTS!$F$11),"B",IF(MAX(E34,F34,G34)&gt;=LISTS!$F$3,"A","B")))))))</f>
-        <v/>
-      </c>
-      <c r="P34" s="14" t="n"/>
-      <c r="Q34" s="14" t="n"/>
-      <c r="R34" s="14">
-        <f>IF(E34="","",IF(B34="","material?",IF(OR(F34="",G34=""),"size?",IF(I34="","exposed Y/N?",IF(H34="","qty?",IF(B34="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S34" s="12">
-        <f t="array" ref="S34">IF(OR(O34="",M34=""),"",IF(B34="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B34&amp;"_"&amp;SUBSTITUTE(O34,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T34" s="12">
-        <f>IF(ISNUMBER(S34),M34*S34,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1" s="59">
+    <row r="33" s="59">
+      <c r="A33" s="133" t="inlineStr">
+        <is>
+          <t>METAL (hollow steel): one line per part, priced PER METRE from the RATES hollow list. MATERIAL = hollow code HOLLOW-&lt;a&gt;x&lt;b&gt;x&lt;wall&gt;, or METAL (= section W x T with RATES!HOLLOW_WALL)</t>
+        </is>
+      </c>
+      <c r="B33" s="134" t="n"/>
+      <c r="C33" s="134" t="n"/>
+      <c r="D33" s="134" t="n"/>
+      <c r="E33" s="134" t="n"/>
+      <c r="F33" s="134" t="n"/>
+      <c r="G33" s="134" t="n"/>
+      <c r="H33" s="134" t="n"/>
+      <c r="I33" s="134" t="n"/>
+      <c r="J33" s="134" t="n"/>
+      <c r="K33" s="134" t="n"/>
+      <c r="L33" s="134" t="n"/>
+      <c r="M33" s="134" t="n"/>
+      <c r="N33" s="134" t="n"/>
+      <c r="O33" s="134" t="n"/>
+      <c r="P33" s="134" t="n"/>
+      <c r="Q33" s="134" t="n"/>
+      <c r="R33" s="134" t="n"/>
+      <c r="S33" s="134" t="n"/>
+      <c r="T33" s="134" t="n"/>
+      <c r="U33" s="134" t="n"/>
+    </row>
+    <row r="34" ht="31.5" customHeight="1" s="59">
+      <c r="A34" s="47" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="B34" s="47" t="inlineStr">
+        <is>
+          <t>MATERIAL / HOLLOW CODE</t>
+        </is>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>LABEL</t>
+        </is>
+      </c>
+      <c r="D34" s="47" t="inlineStr">
+        <is>
+          <t>COMPONENT</t>
+        </is>
+      </c>
+      <c r="E34" s="47" t="inlineStr">
+        <is>
+          <t>L mm</t>
+        </is>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>W mm</t>
+        </is>
+      </c>
+      <c r="G34" s="47" t="inlineStr">
+        <is>
+          <t>T mm</t>
+        </is>
+      </c>
+      <c r="H34" s="47" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="I34" s="47" t="inlineStr">
+        <is>
+          <t>EXPOSED Y/N</t>
+        </is>
+      </c>
+      <c r="J34" s="47" t="n"/>
+      <c r="K34" s="47" t="n"/>
+      <c r="L34" s="47" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="M34" s="47" t="inlineStr">
+        <is>
+          <t>LENGTH m (calc)</t>
+        </is>
+      </c>
+      <c r="N34" s="47" t="inlineStr">
+        <is>
+          <t>FACE m² (calc)</t>
+        </is>
+      </c>
+      <c r="O34" s="47" t="inlineStr">
+        <is>
+          <t>CODE USED (calc)</t>
+        </is>
+      </c>
+      <c r="P34" s="47" t="n"/>
+      <c r="Q34" s="47" t="n"/>
+      <c r="R34" s="47" t="inlineStr">
+        <is>
+          <t>CHECK (calc)</t>
+        </is>
+      </c>
+      <c r="S34" s="47" t="inlineStr">
+        <is>
+          <t>RATE IDR/m (system)</t>
+        </is>
+      </c>
+      <c r="T34" s="47" t="inlineStr">
+        <is>
+          <t>COST IDR (system)</t>
+        </is>
+      </c>
+      <c r="U34" s="135" t="inlineStr">
+        <is>
+          <t>COST USD
+(system)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" s="59">
       <c r="A35" s="9" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="B35" s="10" t="n"/>
       <c r="C35" s="48" t="n"/>
@@ -7307,8 +7349,8 @@
       <c r="J35" s="10" t="n"/>
       <c r="K35" s="10" t="n"/>
       <c r="L35" s="10" t="n"/>
-      <c r="M35" s="25">
-        <f>IF(OR(E35="",F35="",G35=""),"",E35*F35*G35/1000000000*IF(H35="",1,H35))</f>
+      <c r="M35" s="19">
+        <f>IF(E35="","",E35/1000*IF(H35="",1,H35))</f>
         <v/>
       </c>
       <c r="N35" s="19">
@@ -7316,27 +7358,31 @@
         <v/>
       </c>
       <c r="O35" s="14">
-        <f>IF(E35="","",IF(K35&lt;&gt;"",K35,IF(AND(E35*F35*G35/1000000000&lt;LISTS!$F$4,MAX(E35,F35,G35)&lt;LISTS!$F$5),"D",IF(I35="N","C",IF(J35="Y","A-CURVED",IF(AND(MEDIAN(E35,F35,G35)&lt;=LISTS!$F$10,MAX(E35,F35,G35)&lt;=LISTS!$F$11),"B",IF(MAX(E35,F35,G35)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E35="","",IF(UPPER(B35)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F35,G35)&amp;"x"&amp;MAX(F35,G35)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F35,G35)&amp;"x"&amp;MAX(F35,G35)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F35,G35)&amp;"x"&amp;MAX(F35,G35)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F35,G35)&amp;"x"&amp;MAX(F35,G35)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B35),7)="HOLLOW-",UPPER(B35),"HOLLOW-"&amp;B35),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P35" s="14" t="n"/>
       <c r="Q35" s="14" t="n"/>
       <c r="R35" s="14">
-        <f>IF(E35="","",IF(B35="","material?",IF(OR(F35="",G35=""),"size?",IF(I35="","exposed Y/N?",IF(H35="","qty?",IF(B35="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S35" s="12">
-        <f t="array" ref="S35">IF(OR(O35="",M35=""),"",IF(B35="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B35&amp;"_"&amp;SUBSTITUTE(O35,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T35" s="12">
-        <f>IF(ISNUMBER(S35),M35*S35,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1" s="59">
+        <f>IF(E35="","",IF(B35="","material?",IF(OR(F35="",G35=""),"size?",IF(I35="","exposed Y/N?",IF(H35="","qty?",IF(O35="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S35" s="136">
+        <f>IF(E35="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O35,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T35" s="136">
+        <f>IF(AND(ISNUMBER(S35),ISNUMBER(M35)),M35*S35,"")</f>
+        <v/>
+      </c>
+      <c r="U35" s="134">
+        <f>IF(T35="","",T35/RATES!$C$172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" s="59">
       <c r="A36" s="9" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="B36" s="10" t="n"/>
       <c r="C36" s="48" t="n"/>
@@ -7349,8 +7395,8 @@
       <c r="J36" s="10" t="n"/>
       <c r="K36" s="10" t="n"/>
       <c r="L36" s="10" t="n"/>
-      <c r="M36" s="25">
-        <f>IF(OR(E36="",F36="",G36=""),"",E36*F36*G36/1000000000*IF(H36="",1,H36))</f>
+      <c r="M36" s="19">
+        <f>IF(E36="","",E36/1000*IF(H36="",1,H36))</f>
         <v/>
       </c>
       <c r="N36" s="19">
@@ -7358,27 +7404,31 @@
         <v/>
       </c>
       <c r="O36" s="14">
-        <f>IF(E36="","",IF(K36&lt;&gt;"",K36,IF(AND(E36*F36*G36/1000000000&lt;LISTS!$F$4,MAX(E36,F36,G36)&lt;LISTS!$F$5),"D",IF(I36="N","C",IF(J36="Y","A-CURVED",IF(AND(MEDIAN(E36,F36,G36)&lt;=LISTS!$F$10,MAX(E36,F36,G36)&lt;=LISTS!$F$11),"B",IF(MAX(E36,F36,G36)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E36="","",IF(UPPER(B36)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F36,G36)&amp;"x"&amp;MAX(F36,G36)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F36,G36)&amp;"x"&amp;MAX(F36,G36)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F36,G36)&amp;"x"&amp;MAX(F36,G36)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F36,G36)&amp;"x"&amp;MAX(F36,G36)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B36),7)="HOLLOW-",UPPER(B36),"HOLLOW-"&amp;B36),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P36" s="14" t="n"/>
       <c r="Q36" s="14" t="n"/>
       <c r="R36" s="14">
-        <f>IF(E36="","",IF(B36="","material?",IF(OR(F36="",G36=""),"size?",IF(I36="","exposed Y/N?",IF(H36="","qty?",IF(B36="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S36" s="12">
-        <f t="array" ref="S36">IF(OR(O36="",M36=""),"",IF(B36="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B36&amp;"_"&amp;SUBSTITUTE(O36,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T36" s="12">
-        <f>IF(ISNUMBER(S36),M36*S36,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1" s="59">
+        <f>IF(E36="","",IF(B36="","material?",IF(OR(F36="",G36=""),"size?",IF(I36="","exposed Y/N?",IF(H36="","qty?",IF(O36="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S36" s="136">
+        <f>IF(E36="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O36,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T36" s="136">
+        <f>IF(AND(ISNUMBER(S36),ISNUMBER(M36)),M36*S36,"")</f>
+        <v/>
+      </c>
+      <c r="U36" s="134">
+        <f>IF(T36="","",T36/RATES!$C$172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" s="59">
       <c r="A37" s="9" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B37" s="10" t="n"/>
       <c r="C37" s="48" t="n"/>
@@ -7391,8 +7441,8 @@
       <c r="J37" s="10" t="n"/>
       <c r="K37" s="10" t="n"/>
       <c r="L37" s="10" t="n"/>
-      <c r="M37" s="25">
-        <f>IF(OR(E37="",F37="",G37=""),"",E37*F37*G37/1000000000*IF(H37="",1,H37))</f>
+      <c r="M37" s="19">
+        <f>IF(E37="","",E37/1000*IF(H37="",1,H37))</f>
         <v/>
       </c>
       <c r="N37" s="19">
@@ -7400,27 +7450,31 @@
         <v/>
       </c>
       <c r="O37" s="14">
-        <f>IF(E37="","",IF(K37&lt;&gt;"",K37,IF(AND(E37*F37*G37/1000000000&lt;LISTS!$F$4,MAX(E37,F37,G37)&lt;LISTS!$F$5),"D",IF(I37="N","C",IF(J37="Y","A-CURVED",IF(AND(MEDIAN(E37,F37,G37)&lt;=LISTS!$F$10,MAX(E37,F37,G37)&lt;=LISTS!$F$11),"B",IF(MAX(E37,F37,G37)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E37="","",IF(UPPER(B37)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F37,G37)&amp;"x"&amp;MAX(F37,G37)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F37,G37)&amp;"x"&amp;MAX(F37,G37)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F37,G37)&amp;"x"&amp;MAX(F37,G37)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F37,G37)&amp;"x"&amp;MAX(F37,G37)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B37),7)="HOLLOW-",UPPER(B37),"HOLLOW-"&amp;B37),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P37" s="14" t="n"/>
       <c r="Q37" s="14" t="n"/>
       <c r="R37" s="14">
-        <f>IF(E37="","",IF(B37="","material?",IF(OR(F37="",G37=""),"size?",IF(I37="","exposed Y/N?",IF(H37="","qty?",IF(B37="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S37" s="12">
-        <f t="array" ref="S37">IF(OR(O37="",M37=""),"",IF(B37="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B37&amp;"_"&amp;SUBSTITUTE(O37,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T37" s="12">
-        <f>IF(ISNUMBER(S37),M37*S37,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1" s="59">
+        <f>IF(E37="","",IF(B37="","material?",IF(OR(F37="",G37=""),"size?",IF(I37="","exposed Y/N?",IF(H37="","qty?",IF(O37="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S37" s="136">
+        <f>IF(E37="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O37,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T37" s="136">
+        <f>IF(AND(ISNUMBER(S37),ISNUMBER(M37)),M37*S37,"")</f>
+        <v/>
+      </c>
+      <c r="U37" s="134">
+        <f>IF(T37="","",T37/RATES!$C$172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" s="59">
       <c r="A38" s="9" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="B38" s="10" t="n"/>
       <c r="C38" s="48" t="n"/>
@@ -7433,8 +7487,8 @@
       <c r="J38" s="10" t="n"/>
       <c r="K38" s="10" t="n"/>
       <c r="L38" s="10" t="n"/>
-      <c r="M38" s="25">
-        <f>IF(OR(E38="",F38="",G38=""),"",E38*F38*G38/1000000000*IF(H38="",1,H38))</f>
+      <c r="M38" s="19">
+        <f>IF(E38="","",E38/1000*IF(H38="",1,H38))</f>
         <v/>
       </c>
       <c r="N38" s="19">
@@ -7442,27 +7496,31 @@
         <v/>
       </c>
       <c r="O38" s="14">
-        <f>IF(E38="","",IF(K38&lt;&gt;"",K38,IF(AND(E38*F38*G38/1000000000&lt;LISTS!$F$4,MAX(E38,F38,G38)&lt;LISTS!$F$5),"D",IF(I38="N","C",IF(J38="Y","A-CURVED",IF(AND(MEDIAN(E38,F38,G38)&lt;=LISTS!$F$10,MAX(E38,F38,G38)&lt;=LISTS!$F$11),"B",IF(MAX(E38,F38,G38)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E38="","",IF(UPPER(B38)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F38,G38)&amp;"x"&amp;MAX(F38,G38)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F38,G38)&amp;"x"&amp;MAX(F38,G38)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F38,G38)&amp;"x"&amp;MAX(F38,G38)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F38,G38)&amp;"x"&amp;MAX(F38,G38)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B38),7)="HOLLOW-",UPPER(B38),"HOLLOW-"&amp;B38),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P38" s="14" t="n"/>
       <c r="Q38" s="14" t="n"/>
       <c r="R38" s="14">
-        <f>IF(E38="","",IF(B38="","material?",IF(OR(F38="",G38=""),"size?",IF(I38="","exposed Y/N?",IF(H38="","qty?",IF(B38="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S38" s="12">
-        <f t="array" ref="S38">IF(OR(O38="",M38=""),"",IF(B38="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B38&amp;"_"&amp;SUBSTITUTE(O38,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T38" s="12">
-        <f>IF(ISNUMBER(S38),M38*S38,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1" s="59">
+        <f>IF(E38="","",IF(B38="","material?",IF(OR(F38="",G38=""),"size?",IF(I38="","exposed Y/N?",IF(H38="","qty?",IF(O38="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S38" s="136">
+        <f>IF(E38="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O38,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T38" s="136">
+        <f>IF(AND(ISNUMBER(S38),ISNUMBER(M38)),M38*S38,"")</f>
+        <v/>
+      </c>
+      <c r="U38" s="134">
+        <f>IF(T38="","",T38/RATES!$C$172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" s="59">
       <c r="A39" s="9" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B39" s="10" t="n"/>
       <c r="C39" s="48" t="n"/>
@@ -7475,8 +7533,8 @@
       <c r="J39" s="10" t="n"/>
       <c r="K39" s="10" t="n"/>
       <c r="L39" s="10" t="n"/>
-      <c r="M39" s="25">
-        <f>IF(OR(E39="",F39="",G39=""),"",E39*F39*G39/1000000000*IF(H39="",1,H39))</f>
+      <c r="M39" s="19">
+        <f>IF(E39="","",E39/1000*IF(H39="",1,H39))</f>
         <v/>
       </c>
       <c r="N39" s="19">
@@ -7484,27 +7542,31 @@
         <v/>
       </c>
       <c r="O39" s="14">
-        <f>IF(E39="","",IF(K39&lt;&gt;"",K39,IF(AND(E39*F39*G39/1000000000&lt;LISTS!$F$4,MAX(E39,F39,G39)&lt;LISTS!$F$5),"D",IF(I39="N","C",IF(J39="Y","A-CURVED",IF(AND(MEDIAN(E39,F39,G39)&lt;=LISTS!$F$10,MAX(E39,F39,G39)&lt;=LISTS!$F$11),"B",IF(MAX(E39,F39,G39)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E39="","",IF(UPPER(B39)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F39,G39)&amp;"x"&amp;MAX(F39,G39)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F39,G39)&amp;"x"&amp;MAX(F39,G39)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F39,G39)&amp;"x"&amp;MAX(F39,G39)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F39,G39)&amp;"x"&amp;MAX(F39,G39)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B39),7)="HOLLOW-",UPPER(B39),"HOLLOW-"&amp;B39),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P39" s="14" t="n"/>
       <c r="Q39" s="14" t="n"/>
       <c r="R39" s="14">
-        <f>IF(E39="","",IF(B39="","material?",IF(OR(F39="",G39=""),"size?",IF(I39="","exposed Y/N?",IF(H39="","qty?",IF(B39="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S39" s="12">
-        <f t="array" ref="S39">IF(OR(O39="",M39=""),"",IF(B39="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B39&amp;"_"&amp;SUBSTITUTE(O39,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T39" s="12">
-        <f>IF(ISNUMBER(S39),M39*S39,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1" s="59">
+        <f>IF(E39="","",IF(B39="","material?",IF(OR(F39="",G39=""),"size?",IF(I39="","exposed Y/N?",IF(H39="","qty?",IF(O39="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S39" s="136">
+        <f>IF(E39="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O39,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T39" s="136">
+        <f>IF(AND(ISNUMBER(S39),ISNUMBER(M39)),M39*S39,"")</f>
+        <v/>
+      </c>
+      <c r="U39" s="134">
+        <f>IF(T39="","",T39/RATES!$C$172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" s="59">
       <c r="A40" s="9" t="n">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="B40" s="10" t="n"/>
       <c r="C40" s="48" t="n"/>
@@ -7517,8 +7579,8 @@
       <c r="J40" s="10" t="n"/>
       <c r="K40" s="10" t="n"/>
       <c r="L40" s="10" t="n"/>
-      <c r="M40" s="25">
-        <f>IF(OR(E40="",F40="",G40=""),"",E40*F40*G40/1000000000*IF(H40="",1,H40))</f>
+      <c r="M40" s="19">
+        <f>IF(E40="","",E40/1000*IF(H40="",1,H40))</f>
         <v/>
       </c>
       <c r="N40" s="19">
@@ -7526,27 +7588,31 @@
         <v/>
       </c>
       <c r="O40" s="14">
-        <f>IF(E40="","",IF(K40&lt;&gt;"",K40,IF(AND(E40*F40*G40/1000000000&lt;LISTS!$F$4,MAX(E40,F40,G40)&lt;LISTS!$F$5),"D",IF(I40="N","C",IF(J40="Y","A-CURVED",IF(AND(MEDIAN(E40,F40,G40)&lt;=LISTS!$F$10,MAX(E40,F40,G40)&lt;=LISTS!$F$11),"B",IF(MAX(E40,F40,G40)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E40="","",IF(UPPER(B40)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F40,G40)&amp;"x"&amp;MAX(F40,G40)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F40,G40)&amp;"x"&amp;MAX(F40,G40)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F40,G40)&amp;"x"&amp;MAX(F40,G40)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F40,G40)&amp;"x"&amp;MAX(F40,G40)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B40),7)="HOLLOW-",UPPER(B40),"HOLLOW-"&amp;B40),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P40" s="14" t="n"/>
       <c r="Q40" s="14" t="n"/>
       <c r="R40" s="14">
-        <f>IF(E40="","",IF(B40="","material?",IF(OR(F40="",G40=""),"size?",IF(I40="","exposed Y/N?",IF(H40="","qty?",IF(B40="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S40" s="12">
-        <f t="array" ref="S40">IF(OR(O40="",M40=""),"",IF(B40="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B40&amp;"_"&amp;SUBSTITUTE(O40,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T40" s="12">
-        <f>IF(ISNUMBER(S40),M40*S40,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1" s="59">
+        <f>IF(E40="","",IF(B40="","material?",IF(OR(F40="",G40=""),"size?",IF(I40="","exposed Y/N?",IF(H40="","qty?",IF(O40="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S40" s="136">
+        <f>IF(E40="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O40,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T40" s="136">
+        <f>IF(AND(ISNUMBER(S40),ISNUMBER(M40)),M40*S40,"")</f>
+        <v/>
+      </c>
+      <c r="U40" s="134">
+        <f>IF(T40="","",T40/RATES!$C$172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" s="59">
       <c r="A41" s="9" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="B41" s="10" t="n"/>
       <c r="C41" s="48" t="n"/>
@@ -7559,8 +7625,8 @@
       <c r="J41" s="10" t="n"/>
       <c r="K41" s="10" t="n"/>
       <c r="L41" s="10" t="n"/>
-      <c r="M41" s="25">
-        <f>IF(OR(E41="",F41="",G41=""),"",E41*F41*G41/1000000000*IF(H41="",1,H41))</f>
+      <c r="M41" s="19">
+        <f>IF(E41="","",E41/1000*IF(H41="",1,H41))</f>
         <v/>
       </c>
       <c r="N41" s="19">
@@ -7568,27 +7634,31 @@
         <v/>
       </c>
       <c r="O41" s="14">
-        <f>IF(E41="","",IF(K41&lt;&gt;"",K41,IF(AND(E41*F41*G41/1000000000&lt;LISTS!$F$4,MAX(E41,F41,G41)&lt;LISTS!$F$5),"D",IF(I41="N","C",IF(J41="Y","A-CURVED",IF(AND(MEDIAN(E41,F41,G41)&lt;=LISTS!$F$10,MAX(E41,F41,G41)&lt;=LISTS!$F$11),"B",IF(MAX(E41,F41,G41)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E41="","",IF(UPPER(B41)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F41,G41)&amp;"x"&amp;MAX(F41,G41)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F41,G41)&amp;"x"&amp;MAX(F41,G41)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F41,G41)&amp;"x"&amp;MAX(F41,G41)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F41,G41)&amp;"x"&amp;MAX(F41,G41)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B41),7)="HOLLOW-",UPPER(B41),"HOLLOW-"&amp;B41),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P41" s="14" t="n"/>
       <c r="Q41" s="14" t="n"/>
       <c r="R41" s="14">
-        <f>IF(E41="","",IF(B41="","material?",IF(OR(F41="",G41=""),"size?",IF(I41="","exposed Y/N?",IF(H41="","qty?",IF(B41="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S41" s="12">
-        <f t="array" ref="S41">IF(OR(O41="",M41=""),"",IF(B41="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B41&amp;"_"&amp;SUBSTITUTE(O41,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T41" s="12">
-        <f>IF(ISNUMBER(S41),M41*S41,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" ht="15.75" customHeight="1" s="59">
+        <f>IF(E41="","",IF(B41="","material?",IF(OR(F41="",G41=""),"size?",IF(I41="","exposed Y/N?",IF(H41="","qty?",IF(O41="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S41" s="136">
+        <f>IF(E41="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O41,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T41" s="136">
+        <f>IF(AND(ISNUMBER(S41),ISNUMBER(M41)),M41*S41,"")</f>
+        <v/>
+      </c>
+      <c r="U41" s="134">
+        <f>IF(T41="","",T41/RATES!$C$172)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" s="59">
       <c r="A42" s="9" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="B42" s="10" t="n"/>
       <c r="C42" s="48" t="n"/>
@@ -7601,8 +7671,8 @@
       <c r="J42" s="10" t="n"/>
       <c r="K42" s="10" t="n"/>
       <c r="L42" s="10" t="n"/>
-      <c r="M42" s="25">
-        <f>IF(OR(E42="",F42="",G42=""),"",E42*F42*G42/1000000000*IF(H42="",1,H42))</f>
+      <c r="M42" s="19">
+        <f>IF(E42="","",E42/1000*IF(H42="",1,H42))</f>
         <v/>
       </c>
       <c r="N42" s="19">
@@ -7610,21 +7680,25 @@
         <v/>
       </c>
       <c r="O42" s="14">
-        <f>IF(E42="","",IF(K42&lt;&gt;"",K42,IF(AND(E42*F42*G42/1000000000&lt;LISTS!$F$4,MAX(E42,F42,G42)&lt;LISTS!$F$5),"D",IF(I42="N","C",IF(J42="Y","A-CURVED",IF(AND(MEDIAN(E42,F42,G42)&lt;=LISTS!$F$10,MAX(E42,F42,G42)&lt;=LISTS!$F$11),"B",IF(MAX(E42,F42,G42)&gt;=LISTS!$F$3,"A","B")))))))</f>
+        <f>IF(E42="","",IF(UPPER(B42)="METAL",IFERROR(IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F42,G42)&amp;"x"&amp;MAX(F42,G42)&amp;"x"&amp;SUBSTITUTE(RATES!$C$252&amp;"",",","."),RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F42,G42)&amp;"x"&amp;MAX(F42,G42)&amp;"x"&amp;"1",RATES!$A:$A,0)),IFERROR(INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F42,G42)&amp;"x"&amp;MAX(F42,G42)&amp;"x"&amp;"1.2",RATES!$A:$A,0)),INDEX(RATES!$A:$A,MATCH("HOLLOW-"&amp;MIN(F42,G42)&amp;"x"&amp;MAX(F42,G42)&amp;"x"&amp;"1.5",RATES!$A:$A,0))))),"not in list"),IFERROR(INDEX(RATES!$A:$A,MATCH(IF(LEFT(UPPER(B42),7)="HOLLOW-",UPPER(B42),"HOLLOW-"&amp;B42),RATES!$A:$A,0)),"not in list")))</f>
         <v/>
       </c>
       <c r="P42" s="14" t="n"/>
       <c r="Q42" s="14" t="n"/>
       <c r="R42" s="14">
-        <f>IF(E42="","",IF(B42="","material?",IF(OR(F42="",G42=""),"size?",IF(I42="","exposed Y/N?",IF(H42="","qty?",IF(B42="OTHER","OTHER: no rate, price it under hardware","OK"))))))</f>
-        <v/>
-      </c>
-      <c r="S42" s="12">
-        <f t="array" ref="S42">IF(OR(O42="",M42=""),"",IF(B42="MERANTI",RATES!$C$45,IFERROR(INDEX(RATES!$C:$C,MATCH(B42&amp;"_"&amp;SUBSTITUTE(O42,"-CURVED","C"),RATES!$A:$A,0)),"rate?")))</f>
-        <v/>
-      </c>
-      <c r="T42" s="12">
-        <f>IF(ISNUMBER(S42),M42*S42,"")</f>
+        <f>IF(E42="","",IF(B42="","material?",IF(OR(F42="",G42=""),"size?",IF(I42="","exposed Y/N?",IF(H42="","qty?",IF(O42="not in list","hollow code?","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="S42" s="136">
+        <f>IF(E42="","",IFERROR(INDEX(RATES!$C:$C,MATCH(O42,RATES!$A:$A,0)),"rate?"))</f>
+        <v/>
+      </c>
+      <c r="T42" s="136">
+        <f>IF(AND(ISNUMBER(S42),ISNUMBER(M42)),M42*S42,"")</f>
+        <v/>
+      </c>
+      <c r="U42" s="134">
+        <f>IF(T42="","",T42/RATES!$C$172)</f>
         <v/>
       </c>
     </row>
@@ -8941,7 +9015,22 @@
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1" s="59"/>
-    <row r="80" ht="15.75" customHeight="1" s="59"/>
+    <row r="80" ht="15.75" customHeight="1" s="59">
+      <c r="C80" s="137" t="inlineStr">
+        <is>
+          <t>METAL (hollow, per m)</t>
+        </is>
+      </c>
+      <c r="D80" s="137">
+        <f>SUM(T35:T42)</f>
+        <v/>
+      </c>
+      <c r="F80" s="137" t="inlineStr">
+        <is>
+          <t>Σ length m × IDR/m of the hollow code (RATES list)</t>
+        </is>
+      </c>
+    </row>
     <row r="81" ht="15.75" customHeight="1" s="59">
       <c r="A81" s="5" t="inlineStr">
         <is>
@@ -8961,7 +9050,7 @@
         </is>
       </c>
       <c r="D82" s="25">
-        <f>SUM(M18:M42)</f>
+        <f>SUM(M18:M32)</f>
         <v/>
       </c>
     </row>
@@ -8983,7 +9072,7 @@
         </is>
       </c>
       <c r="D84" s="19">
-        <f>SUMIF(I18:I42,"Y",N18:N42)+SUMIF(I46:I60,1,N46:N60)+2*SUMIF(I46:I60,2,N46:N60)</f>
+        <f>SUMIF(I18:I32,"Y",N18:N32)+SUMIF(I35:I42,"Y",N35:N42)+SUMIF(I46:I60,1,N46:N60)+2*SUMIF(I46:I60,2,N46:N60)</f>
         <v/>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -9021,7 +9110,7 @@
         </is>
       </c>
       <c r="D87" s="12">
-        <f>SUM(T18:T42)</f>
+        <f>SUM(T18:T32)</f>
         <v/>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -9165,8 +9254,13 @@
         </is>
       </c>
       <c r="D96" s="16">
-        <f>SUM(D87:D95)</f>
-        <v/>
+        <f>SUM(D87:D95)+D80</f>
+        <v/>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>timber + metal + fasteners + panels + finishing + hardware + packing</t>
+        </is>
       </c>
     </row>
     <row r="97" ht="15.75" customHeight="1" s="59">
@@ -9241,7 +9335,7 @@
         </is>
       </c>
       <c r="D102" s="40">
-        <f>COUNTIF(R18:R42,"?*")-COUNTIF(R18:R42,"OK")+COUNTIF(R46:R60,"?*")-COUNTIF(R46:R60,"OK")+COUNTIF(S18:S60,"rate?")</f>
+        <f>COUNTIF(R18:R32,"?*")-COUNTIF(R18:R32,"OK")+COUNTIF(R35:R42,"?*")-COUNTIF(R35:R42,"OK")+COUNTIF(R46:R60,"?*")-COUNTIF(R46:R60,"OK")+COUNTIF(S18:S60,"rate?")</f>
         <v/>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -10224,13 +10318,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="K18:K42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K18:K32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A,A-CURVED,B,C,D"</formula1>
     </dataValidation>
     <dataValidation sqref="I46:I60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"0,1,2"</formula1>
     </dataValidation>
-    <dataValidation sqref="C6 I18:J42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pilih dari daftar" error="Nilai di luar daftar; pilih dari dropdown agar rumus mengenalinya." type="list" errorStyle="warning">
+    <dataValidation sqref="C6 I18:J32 I35:I42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pilih dari daftar" error="Nilai di luar daftar; pilih dari dropdown agar rumus mengenalinya." type="list" errorStyle="warning">
       <formula1>"Y,N"</formula1>
     </dataValidation>
     <dataValidation sqref="B64:B78" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Pilih dari daftar" error="Nilai di luar daftar; pilih dari dropdown agar rumus mengenalinya." type="list" errorStyle="warning">

</xml_diff>

<commit_message>
Rates+summary revisi 23 Okt: Mindi A-D baru, MISC 4%, OH_PCT dihapus, summary = TOTAL/MISC/DIRECT(HPP)/USD/TARGET (x1.5), kurs summary 17800 (FX_TARGET)
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
@@ -29,6 +29,7 @@
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
     <numFmt numFmtId="169" formatCode="0.0%"/>
     <numFmt numFmtId="170" formatCode="[$Rp]#,##0"/>
+    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -393,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="140">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -654,6 +655,10 @@
     </xf>
     <xf numFmtId="3" fontId="2" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="2" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2334,12 +2339,12 @@
       </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
-          <t>MISC + OVERHEAD</t>
+          <t>MISC 4%</t>
         </is>
       </c>
       <c r="Q4" s="8" t="inlineStr">
         <is>
-          <t>UNIT COST IDR</t>
+          <t>DIRECT COST IDR (HPP)</t>
         </is>
       </c>
       <c r="R4" s="8" t="inlineStr">
@@ -2483,11 +2488,11 @@
         <v/>
       </c>
       <c r="P6" s="12">
-        <f>IF(OR($J6="",$J6="no tab yet",$J6="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C6&amp;"'!D97")+INDIRECT("'"&amp;$C6&amp;"'!D98"),""))</f>
+        <f>IF(OR($J6="",$J6="no tab yet",$J6="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C6&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q6" s="16">
-        <f>IF(OR($J6="",$J6="no tab yet",$J6="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C6&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J6="",$J6="no tab yet",$J6="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C6&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R6" s="12">
@@ -3221,11 +3226,11 @@
         <v/>
       </c>
       <c r="P30" s="12">
-        <f>IF(OR($J30="",$J30="no tab yet",$J30="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C30&amp;"'!D97")+INDIRECT("'"&amp;$C30&amp;"'!D98"),""))</f>
+        <f>IF(OR($J30="",$J30="no tab yet",$J30="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C30&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q30" s="16">
-        <f>IF(OR($J30="",$J30="no tab yet",$J30="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C30&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J30="",$J30="no tab yet",$J30="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C30&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R30" s="12">
@@ -3292,11 +3297,11 @@
         <v/>
       </c>
       <c r="P31" s="12">
-        <f>IF(OR($J31="",$J31="no tab yet",$J31="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C31&amp;"'!D97")+INDIRECT("'"&amp;$C31&amp;"'!D98"),""))</f>
+        <f>IF(OR($J31="",$J31="no tab yet",$J31="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C31&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q31" s="16">
-        <f>IF(OR($J31="",$J31="no tab yet",$J31="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C31&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J31="",$J31="no tab yet",$J31="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C31&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R31" s="12">
@@ -3363,11 +3368,11 @@
         <v/>
       </c>
       <c r="P32" s="12">
-        <f>IF(OR($J32="",$J32="no tab yet",$J32="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C32&amp;"'!D97")+INDIRECT("'"&amp;$C32&amp;"'!D98"),""))</f>
+        <f>IF(OR($J32="",$J32="no tab yet",$J32="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C32&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q32" s="16">
-        <f>IF(OR($J32="",$J32="no tab yet",$J32="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C32&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J32="",$J32="no tab yet",$J32="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C32&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R32" s="12">
@@ -3434,11 +3439,11 @@
         <v/>
       </c>
       <c r="P33" s="12">
-        <f>IF(OR($J33="",$J33="no tab yet",$J33="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C33&amp;"'!D97")+INDIRECT("'"&amp;$C33&amp;"'!D98"),""))</f>
+        <f>IF(OR($J33="",$J33="no tab yet",$J33="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C33&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q33" s="16">
-        <f>IF(OR($J33="",$J33="no tab yet",$J33="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C33&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J33="",$J33="no tab yet",$J33="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C33&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R33" s="12">
@@ -3505,11 +3510,11 @@
         <v/>
       </c>
       <c r="P34" s="12">
-        <f>IF(OR($J34="",$J34="no tab yet",$J34="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C34&amp;"'!D97")+INDIRECT("'"&amp;$C34&amp;"'!D98"),""))</f>
+        <f>IF(OR($J34="",$J34="no tab yet",$J34="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C34&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q34" s="16">
-        <f>IF(OR($J34="",$J34="no tab yet",$J34="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C34&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J34="",$J34="no tab yet",$J34="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C34&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R34" s="12">
@@ -3576,11 +3581,11 @@
         <v/>
       </c>
       <c r="P35" s="12">
-        <f>IF(OR($J35="",$J35="no tab yet",$J35="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C35&amp;"'!D97")+INDIRECT("'"&amp;$C35&amp;"'!D98"),""))</f>
+        <f>IF(OR($J35="",$J35="no tab yet",$J35="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C35&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q35" s="16">
-        <f>IF(OR($J35="",$J35="no tab yet",$J35="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C35&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J35="",$J35="no tab yet",$J35="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C35&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R35" s="12">
@@ -3647,11 +3652,11 @@
         <v/>
       </c>
       <c r="P36" s="12">
-        <f>IF(OR($J36="",$J36="no tab yet",$J36="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C36&amp;"'!D97")+INDIRECT("'"&amp;$C36&amp;"'!D98"),""))</f>
+        <f>IF(OR($J36="",$J36="no tab yet",$J36="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C36&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q36" s="16">
-        <f>IF(OR($J36="",$J36="no tab yet",$J36="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C36&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J36="",$J36="no tab yet",$J36="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C36&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R36" s="12">
@@ -3718,11 +3723,11 @@
         <v/>
       </c>
       <c r="P37" s="12">
-        <f>IF(OR($J37="",$J37="no tab yet",$J37="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C37&amp;"'!D97")+INDIRECT("'"&amp;$C37&amp;"'!D98"),""))</f>
+        <f>IF(OR($J37="",$J37="no tab yet",$J37="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C37&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q37" s="16">
-        <f>IF(OR($J37="",$J37="no tab yet",$J37="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C37&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J37="",$J37="no tab yet",$J37="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C37&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R37" s="12">
@@ -3789,11 +3794,11 @@
         <v/>
       </c>
       <c r="P38" s="12">
-        <f>IF(OR($J38="",$J38="no tab yet",$J38="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C38&amp;"'!D97")+INDIRECT("'"&amp;$C38&amp;"'!D98"),""))</f>
+        <f>IF(OR($J38="",$J38="no tab yet",$J38="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C38&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q38" s="16">
-        <f>IF(OR($J38="",$J38="no tab yet",$J38="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C38&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J38="",$J38="no tab yet",$J38="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C38&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R38" s="12">
@@ -3860,11 +3865,11 @@
         <v/>
       </c>
       <c r="P39" s="12">
-        <f>IF(OR($J39="",$J39="no tab yet",$J39="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C39&amp;"'!D97")+INDIRECT("'"&amp;$C39&amp;"'!D98"),""))</f>
+        <f>IF(OR($J39="",$J39="no tab yet",$J39="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C39&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q39" s="16">
-        <f>IF(OR($J39="",$J39="no tab yet",$J39="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C39&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J39="",$J39="no tab yet",$J39="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C39&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R39" s="12">
@@ -3931,11 +3936,11 @@
         <v/>
       </c>
       <c r="P40" s="12">
-        <f>IF(OR($J40="",$J40="no tab yet",$J40="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C40&amp;"'!D97")+INDIRECT("'"&amp;$C40&amp;"'!D98"),""))</f>
+        <f>IF(OR($J40="",$J40="no tab yet",$J40="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C40&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q40" s="16">
-        <f>IF(OR($J40="",$J40="no tab yet",$J40="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C40&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J40="",$J40="no tab yet",$J40="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C40&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R40" s="12">
@@ -4002,11 +4007,11 @@
         <v/>
       </c>
       <c r="P41" s="12">
-        <f>IF(OR($J41="",$J41="no tab yet",$J41="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C41&amp;"'!D97")+INDIRECT("'"&amp;$C41&amp;"'!D98"),""))</f>
+        <f>IF(OR($J41="",$J41="no tab yet",$J41="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C41&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q41" s="16">
-        <f>IF(OR($J41="",$J41="no tab yet",$J41="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C41&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J41="",$J41="no tab yet",$J41="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C41&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R41" s="12">
@@ -4073,11 +4078,11 @@
         <v/>
       </c>
       <c r="P42" s="12">
-        <f>IF(OR($J42="",$J42="no tab yet",$J42="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C42&amp;"'!D97")+INDIRECT("'"&amp;$C42&amp;"'!D98"),""))</f>
+        <f>IF(OR($J42="",$J42="no tab yet",$J42="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C42&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q42" s="16">
-        <f>IF(OR($J42="",$J42="no tab yet",$J42="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C42&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J42="",$J42="no tab yet",$J42="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C42&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R42" s="12">
@@ -4144,11 +4149,11 @@
         <v/>
       </c>
       <c r="P43" s="12">
-        <f>IF(OR($J43="",$J43="no tab yet",$J43="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C43&amp;"'!D97")+INDIRECT("'"&amp;$C43&amp;"'!D98"),""))</f>
+        <f>IF(OR($J43="",$J43="no tab yet",$J43="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C43&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q43" s="16">
-        <f>IF(OR($J43="",$J43="no tab yet",$J43="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C43&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J43="",$J43="no tab yet",$J43="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C43&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R43" s="12">
@@ -4215,11 +4220,11 @@
         <v/>
       </c>
       <c r="P44" s="12">
-        <f>IF(OR($J44="",$J44="no tab yet",$J44="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C44&amp;"'!D97")+INDIRECT("'"&amp;$C44&amp;"'!D98"),""))</f>
+        <f>IF(OR($J44="",$J44="no tab yet",$J44="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C44&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q44" s="16">
-        <f>IF(OR($J44="",$J44="no tab yet",$J44="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C44&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J44="",$J44="no tab yet",$J44="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C44&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R44" s="12">
@@ -4286,11 +4291,11 @@
         <v/>
       </c>
       <c r="P45" s="12">
-        <f>IF(OR($J45="",$J45="no tab yet",$J45="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C45&amp;"'!D97")+INDIRECT("'"&amp;$C45&amp;"'!D98"),""))</f>
+        <f>IF(OR($J45="",$J45="no tab yet",$J45="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C45&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q45" s="16">
-        <f>IF(OR($J45="",$J45="no tab yet",$J45="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C45&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J45="",$J45="no tab yet",$J45="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C45&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R45" s="12">
@@ -4357,11 +4362,11 @@
         <v/>
       </c>
       <c r="P46" s="12">
-        <f>IF(OR($J46="",$J46="no tab yet",$J46="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C46&amp;"'!D97")+INDIRECT("'"&amp;$C46&amp;"'!D98"),""))</f>
+        <f>IF(OR($J46="",$J46="no tab yet",$J46="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C46&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q46" s="16">
-        <f>IF(OR($J46="",$J46="no tab yet",$J46="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C46&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J46="",$J46="no tab yet",$J46="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C46&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R46" s="12">
@@ -4428,11 +4433,11 @@
         <v/>
       </c>
       <c r="P47" s="12">
-        <f>IF(OR($J47="",$J47="no tab yet",$J47="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C47&amp;"'!D97")+INDIRECT("'"&amp;$C47&amp;"'!D98"),""))</f>
+        <f>IF(OR($J47="",$J47="no tab yet",$J47="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C47&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q47" s="16">
-        <f>IF(OR($J47="",$J47="no tab yet",$J47="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C47&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J47="",$J47="no tab yet",$J47="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C47&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R47" s="12">
@@ -4499,11 +4504,11 @@
         <v/>
       </c>
       <c r="P48" s="12">
-        <f>IF(OR($J48="",$J48="no tab yet",$J48="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C48&amp;"'!D97")+INDIRECT("'"&amp;$C48&amp;"'!D98"),""))</f>
+        <f>IF(OR($J48="",$J48="no tab yet",$J48="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C48&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q48" s="16">
-        <f>IF(OR($J48="",$J48="no tab yet",$J48="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C48&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J48="",$J48="no tab yet",$J48="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C48&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R48" s="12">
@@ -4570,11 +4575,11 @@
         <v/>
       </c>
       <c r="P49" s="12">
-        <f>IF(OR($J49="",$J49="no tab yet",$J49="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C49&amp;"'!D97")+INDIRECT("'"&amp;$C49&amp;"'!D98"),""))</f>
+        <f>IF(OR($J49="",$J49="no tab yet",$J49="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C49&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q49" s="16">
-        <f>IF(OR($J49="",$J49="no tab yet",$J49="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C49&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J49="",$J49="no tab yet",$J49="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C49&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R49" s="12">
@@ -4641,11 +4646,11 @@
         <v/>
       </c>
       <c r="P50" s="12">
-        <f>IF(OR($J50="",$J50="no tab yet",$J50="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C50&amp;"'!D97")+INDIRECT("'"&amp;$C50&amp;"'!D98"),""))</f>
+        <f>IF(OR($J50="",$J50="no tab yet",$J50="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C50&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q50" s="16">
-        <f>IF(OR($J50="",$J50="no tab yet",$J50="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C50&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J50="",$J50="no tab yet",$J50="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C50&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R50" s="12">
@@ -4712,11 +4717,11 @@
         <v/>
       </c>
       <c r="P51" s="12">
-        <f>IF(OR($J51="",$J51="no tab yet",$J51="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C51&amp;"'!D97")+INDIRECT("'"&amp;$C51&amp;"'!D98"),""))</f>
+        <f>IF(OR($J51="",$J51="no tab yet",$J51="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C51&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q51" s="16">
-        <f>IF(OR($J51="",$J51="no tab yet",$J51="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C51&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J51="",$J51="no tab yet",$J51="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C51&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R51" s="12">
@@ -4783,11 +4788,11 @@
         <v/>
       </c>
       <c r="P52" s="12">
-        <f>IF(OR($J52="",$J52="no tab yet",$J52="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C52&amp;"'!D97")+INDIRECT("'"&amp;$C52&amp;"'!D98"),""))</f>
+        <f>IF(OR($J52="",$J52="no tab yet",$J52="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C52&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q52" s="16">
-        <f>IF(OR($J52="",$J52="no tab yet",$J52="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C52&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J52="",$J52="no tab yet",$J52="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C52&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R52" s="12">
@@ -4854,11 +4859,11 @@
         <v/>
       </c>
       <c r="P53" s="12">
-        <f>IF(OR($J53="",$J53="no tab yet",$J53="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C53&amp;"'!D97")+INDIRECT("'"&amp;$C53&amp;"'!D98"),""))</f>
+        <f>IF(OR($J53="",$J53="no tab yet",$J53="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C53&amp;"'!D97"),""))</f>
         <v/>
       </c>
       <c r="Q53" s="16">
-        <f>IF(OR($J53="",$J53="no tab yet",$J53="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C53&amp;"'!D99")+0,""))</f>
+        <f>IF(OR($J53="",$J53="no tab yet",$J53="tab empty"),"",IFERROR(INDIRECT("'"&amp;$C53&amp;"'!D98")+0,""))</f>
         <v/>
       </c>
       <c r="R53" s="12">
@@ -9250,23 +9255,23 @@
     <row r="96" ht="15.75" customHeight="1" s="59">
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>DIRECT COST</t>
+          <t>TOTAL COST</t>
         </is>
       </c>
       <c r="D96" s="16">
-        <f>SUM(D87:D95)+D80</f>
+        <f>SUM(D87:D95)</f>
         <v/>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>timber + metal + fasteners + panels + finishing + hardware + packing</t>
+          <t>Σ of the nine lines above</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15.75" customHeight="1" s="59">
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>MISC 5%</t>
+          <t>MISC 4%</t>
         </is>
       </c>
       <c r="D97" s="12">
@@ -9275,56 +9280,70 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>direct × MISC_PCT</t>
+          <t>total cost × MISC_PCT</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="59">
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>OVERHEAD</t>
-        </is>
-      </c>
-      <c r="D98" s="12">
-        <f>(D96+D97)*RATES!$C$55</f>
-        <v/>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>(direct + misc) × OH_PCT</t>
+          <t>DIRECT COST IDR (HPP)</t>
+        </is>
+      </c>
+      <c r="D98" s="16">
+        <f>D96+D97</f>
+        <v/>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>total cost + misc</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1" s="59">
+      <c r="B99" s="132">
+        <f>RATES!$C$169</f>
+        <v/>
+      </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>UNIT COST IDR</t>
-        </is>
-      </c>
-      <c r="D99" s="16">
-        <f>D96+D97+D98</f>
-        <v/>
+          <t>DIRECT COST USD</t>
+        </is>
+      </c>
+      <c r="D99" s="138">
+        <f>D98/RATES!$C$169</f>
+        <v/>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>HPP ÷ FX_TARGET (IDR/USD in column B)</t>
+        </is>
       </c>
     </row>
     <row r="100" ht="15.75" customHeight="1" s="59">
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Carton board m² (6 sides)</t>
-        </is>
-      </c>
-      <c r="D100" s="19">
-        <f>L15</f>
-        <v/>
+          <t>TARGET PRICE USD</t>
+        </is>
+      </c>
+      <c r="D100" s="138">
+        <f>D99*RATES!$C$55</f>
+        <v/>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>direct cost USD × TARGET_X</t>
+        </is>
       </c>
     </row>
     <row r="101" ht="15.75" customHeight="1" s="59">
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>ORDER QTY × UNIT COST</t>
+          <t>ORDER QTY × DIRECT COST IDR</t>
         </is>
       </c>
       <c r="D101" s="16">
-        <f>IF(ISNUMBER(C4),C4,0)*D99</f>
+        <f>IF(ISNUMBER(C4),C4,0)*D98</f>
         <v/>
       </c>
     </row>
@@ -11421,7 +11440,7 @@
         </is>
       </c>
       <c r="C40" s="108" t="n">
-        <v>18057965.09</v>
+        <v>11918256.96</v>
       </c>
       <c r="D40" s="96" t="inlineStr">
         <is>
@@ -11446,7 +11465,7 @@
         </is>
       </c>
       <c r="C41" s="108" t="n">
-        <v>21620953.31</v>
+        <v>14269829.18</v>
       </c>
       <c r="D41" s="96" t="inlineStr">
         <is>
@@ -11471,7 +11490,7 @@
         </is>
       </c>
       <c r="C42" s="108" t="n">
-        <v>14818884.89</v>
+        <v>9780464.027000001</v>
       </c>
       <c r="D42" s="96" t="inlineStr">
         <is>
@@ -11496,7 +11515,7 @@
         </is>
       </c>
       <c r="C43" s="108" t="n">
-        <v>13199344.79</v>
+        <v>8711567.561000001</v>
       </c>
       <c r="D43" s="96" t="inlineStr">
         <is>
@@ -11521,7 +11540,7 @@
         </is>
       </c>
       <c r="C44" s="108" t="n">
-        <v>11579804.69</v>
+        <v>7642671.095</v>
       </c>
       <c r="D44" s="96" t="inlineStr">
         <is>
@@ -11787,7 +11806,7 @@
         </is>
       </c>
       <c r="C54" s="106" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="D54" s="96" t="inlineStr">
         <is>
@@ -11796,7 +11815,7 @@
       </c>
       <c r="E54" s="96" t="inlineStr">
         <is>
-          <t>Decision 29 Sep</t>
+          <t>Rizky 23 Okt 2026: 4% of TOTAL COST (was 5%)</t>
         </is>
       </c>
       <c r="F54" s="95" t="n"/>
@@ -11807,26 +11826,25 @@
     <row r="55">
       <c r="A55" s="102" t="inlineStr">
         <is>
-          <t>OH_PCT</t>
+          <t>TARGET_X</t>
         </is>
       </c>
       <c r="B55" s="103" t="inlineStr">
         <is>
-          <t>Overhead, × (direct + misc)</t>
-        </is>
-      </c>
-      <c r="C55" s="110">
-        <f>$C$26/$C$27</f>
-        <v/>
+          <t>Target price = DIRECT COST in USD x this factor</t>
+        </is>
+      </c>
+      <c r="C55" s="139" t="n">
+        <v>1.5</v>
       </c>
       <c r="D55" s="96" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>x</t>
         </is>
       </c>
       <c r="E55" s="96" t="inlineStr">
         <is>
-          <t>Overhead pool ÷ STMV direct cost</t>
+          <t>Rizky 23 Okt 2026 (replaces OH_PCT, deleted). Blue = input</t>
         </is>
       </c>
       <c r="F55" s="95" t="n"/>
@@ -14737,7 +14755,33 @@
       <c r="H168" s="95" t="n"/>
       <c r="I168" s="95" t="n"/>
     </row>
-    <row r="169"/>
+    <row r="169">
+      <c r="A169" s="113" t="inlineStr">
+        <is>
+          <t>FX_TARGET</t>
+        </is>
+      </c>
+      <c r="B169" s="117" t="inlineStr">
+        <is>
+          <t>USD rate for the summary USD lines, ITEMS USD columns and target price</t>
+        </is>
+      </c>
+      <c r="C169" s="114" t="n">
+        <v>17800</v>
+      </c>
+      <c r="D169" s="113" t="inlineStr">
+        <is>
+          <t>IDR/USD</t>
+        </is>
+      </c>
+      <c r="E169" s="113" t="inlineStr">
+        <is>
+          <t>Rizky 23 Okt 2026. Hardware/board quotes still use FX_USD (row 172)</t>
+        </is>
+      </c>
+      <c r="F169" s="95" t="n"/>
+      <c r="G169" s="95" t="n"/>
+    </row>
     <row r="170">
       <c r="A170" s="97" t="inlineStr">
         <is>
@@ -14948,7 +14992,6 @@
       <c r="H176" s="95" t="n"/>
       <c r="I176" s="95" t="n"/>
     </row>
-    <row r="177"/>
     <row r="178">
       <c r="A178" s="119" t="inlineStr">
         <is>
@@ -16469,7 +16512,6 @@
         <v>933</v>
       </c>
     </row>
-    <row r="216"/>
     <row r="217">
       <c r="A217" s="97" t="inlineStr">
         <is>
@@ -16773,7 +16815,6 @@
       <c r="H225" s="95" t="n"/>
       <c r="I225" s="95" t="n"/>
     </row>
-    <row r="226"/>
     <row r="227">
       <c r="A227" s="97" t="inlineStr">
         <is>
@@ -16867,7 +16908,6 @@
       <c r="H229" s="95" t="n"/>
       <c r="I229" s="95" t="n"/>
     </row>
-    <row r="230"/>
     <row r="231">
       <c r="A231" s="127" t="inlineStr">
         <is>
@@ -17351,7 +17391,6 @@
       <c r="H249" s="95" t="n"/>
       <c r="I249" s="95" t="n"/>
     </row>
-    <row r="250"/>
     <row r="251">
       <c r="A251" s="127" t="inlineStr">
         <is>
@@ -36929,6 +36968,11 @@
           <t>SUMMARY (system): cost per ONE item, from the RATES tab. Do not type here.</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>COST USD (system)</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15.75" customHeight="1" s="59">
       <c r="C82" s="5" t="inlineStr">
@@ -37137,18 +37181,23 @@
     <row r="96" ht="15.75" customHeight="1" s="59">
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>DIRECT COST</t>
+          <t>TOTAL COST</t>
         </is>
       </c>
       <c r="D96" s="16">
         <f>SUM(D87:D95)</f>
         <v/>
       </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Σ of the nine lines above</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15.75" customHeight="1" s="59">
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>MISC 5%</t>
+          <t>MISC 4%</t>
         </is>
       </c>
       <c r="D97" s="12">
@@ -37157,56 +37206,70 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>direct × MISC_PCT</t>
+          <t>total cost × MISC_PCT</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="59">
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>OVERHEAD</t>
-        </is>
-      </c>
-      <c r="D98" s="12">
-        <f>(D96+D97)*RATES!$C$55</f>
-        <v/>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>(direct + misc) × OH_PCT</t>
+          <t>DIRECT COST IDR (HPP)</t>
+        </is>
+      </c>
+      <c r="D98" s="16">
+        <f>D96+D97</f>
+        <v/>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>total cost + misc</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1" s="59">
+      <c r="B99" s="132">
+        <f>RATES!$C$169</f>
+        <v/>
+      </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>UNIT COST IDR</t>
-        </is>
-      </c>
-      <c r="D99" s="16">
-        <f>D96+D97+D98</f>
-        <v/>
+          <t>DIRECT COST USD</t>
+        </is>
+      </c>
+      <c r="D99" s="138">
+        <f>D98/RATES!$C$169</f>
+        <v/>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>HPP ÷ FX_TARGET (IDR/USD in column B)</t>
+        </is>
       </c>
     </row>
     <row r="100" ht="15.75" customHeight="1" s="59">
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Carton board m² (6 sides)</t>
-        </is>
-      </c>
-      <c r="D100" s="19">
-        <f>L15</f>
-        <v/>
+          <t>TARGET PRICE USD</t>
+        </is>
+      </c>
+      <c r="D100" s="138">
+        <f>D99*RATES!$C$55</f>
+        <v/>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>direct cost USD × TARGET_X</t>
+        </is>
       </c>
     </row>
     <row r="101" ht="15.75" customHeight="1" s="59">
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>ORDER QTY × UNIT COST</t>
+          <t>ORDER QTY × DIRECT COST IDR</t>
         </is>
       </c>
       <c r="D101" s="16">
-        <f>IF(ISNUMBER(C4),C4,0)*D99</f>
+        <f>IF(ISNUMBER(C4),C4,0)*D98</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Napier: konstruksi standar Tala (karkas panel 301/306/302/601, laci rumus pabrik, tanpa rail kecil) untuk 7 item kotak; tabel item lebih rapat, NOTE di paling kanan, COST USD berformat
</commit_message>
<xml_diff>
--- a/data/GOLDEN_MASTER.xlsx
+++ b/data/GOLDEN_MASTER.xlsx
@@ -9339,7 +9339,7 @@
     <row r="101" ht="15.75" customHeight="1" s="59">
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>ORDER QTY × DIRECT COST IDR</t>
+          <t>ORDER QTY × HPP IDR</t>
         </is>
       </c>
       <c r="D101" s="16">
@@ -37265,7 +37265,7 @@
     <row r="101" ht="15.75" customHeight="1" s="59">
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>ORDER QTY × DIRECT COST IDR</t>
+          <t>ORDER QTY × HPP IDR</t>
         </is>
       </c>
       <c r="D101" s="16">

</xml_diff>